<commit_message>
Refactor: Adjust text element column boundaries and order in prompt data for improved parsing.
</commit_message>
<xml_diff>
--- a/data/out/sample/001317375.xlsx
+++ b/data/out/sample/001317375.xlsx
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -194,12 +194,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -207,12 +202,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -228,6 +217,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -238,6 +229,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -921,7 +915,7 @@
       <c r="AL7" s="9" t="n"/>
       <c r="AM7" s="8" t="inlineStr">
         <is>
-          <t>△△△△</t>
+          <t>□□□□</t>
         </is>
       </c>
       <c r="AN7" s="9" t="n"/>
@@ -1274,7 +1268,7 @@
       <c r="AU12" s="9" t="n"/>
       <c r="AV12" s="9" t="n"/>
       <c r="AW12" s="9" t="n"/>
-      <c r="AX12" s="10" t="n"/>
+      <c r="AX12" s="12" t="n"/>
       <c r="AY12" s="9" t="n"/>
       <c r="AZ12" s="9" t="n"/>
       <c r="BA12" s="9" t="n"/>
@@ -1402,7 +1396,7 @@
       <c r="AU13" s="13" t="n"/>
       <c r="AV13" s="13" t="n"/>
       <c r="AW13" s="13" t="n"/>
-      <c r="AX13" s="10" t="n"/>
+      <c r="AX13" s="12" t="n"/>
       <c r="AY13" s="9" t="n"/>
       <c r="AZ13" s="11" t="inlineStr">
         <is>
@@ -1411,7 +1405,7 @@
       </c>
       <c r="BA13" s="9" t="n"/>
       <c r="BB13" s="9" t="n"/>
-      <c r="BC13" s="9" t="n"/>
+      <c r="BC13" s="12" t="n"/>
       <c r="BD13" s="9" t="n"/>
       <c r="BE13" s="11" t="inlineStr">
         <is>
@@ -1421,7 +1415,7 @@
       <c r="BF13" s="9" t="n"/>
       <c r="BG13" s="9" t="n"/>
       <c r="BH13" s="9" t="n"/>
-      <c r="BI13" s="9" t="n"/>
+      <c r="BI13" s="12" t="n"/>
       <c r="BJ13" s="9" t="n"/>
       <c r="BK13" s="11" t="inlineStr">
         <is>
@@ -1430,7 +1424,7 @@
       </c>
       <c r="BL13" s="9" t="n"/>
       <c r="BM13" s="9" t="n"/>
-      <c r="BN13" s="17" t="n"/>
+      <c r="BN13" s="12" t="n"/>
       <c r="BO13" s="9" t="n"/>
       <c r="BP13" s="9" t="n"/>
       <c r="BQ13" s="11" t="inlineStr">
@@ -1440,7 +1434,7 @@
       </c>
       <c r="BR13" s="9" t="n"/>
       <c r="BS13" s="9" t="n"/>
-      <c r="BT13" s="9" t="n"/>
+      <c r="BT13" s="12" t="n"/>
       <c r="BU13" s="9" t="n"/>
       <c r="BV13" s="11" t="inlineStr">
         <is>
@@ -1450,7 +1444,7 @@
       <c r="BW13" s="9" t="n"/>
       <c r="BX13" s="9" t="n"/>
       <c r="BY13" s="9" t="n"/>
-      <c r="BZ13" s="9" t="n"/>
+      <c r="BZ13" s="12" t="n"/>
       <c r="CA13" s="9" t="n"/>
       <c r="CB13" s="11" t="inlineStr">
         <is>
@@ -1469,7 +1463,7 @@
       <c r="CH13" s="9" t="n"/>
       <c r="CI13" s="9" t="n"/>
       <c r="CJ13" s="9" t="n"/>
-      <c r="CK13" s="9" t="n"/>
+      <c r="CK13" s="12" t="n"/>
       <c r="CL13" s="9" t="n"/>
       <c r="CM13" s="11" t="inlineStr">
         <is>
@@ -1479,7 +1473,7 @@
       <c r="CN13" s="9" t="n"/>
       <c r="CO13" s="9" t="n"/>
       <c r="CP13" s="9" t="n"/>
-      <c r="CQ13" s="9" t="n"/>
+      <c r="CQ13" s="12" t="n"/>
       <c r="CR13" s="9" t="n"/>
       <c r="CS13" s="11" t="inlineStr">
         <is>
@@ -1488,7 +1482,7 @@
       </c>
       <c r="CT13" s="9" t="n"/>
       <c r="CU13" s="9" t="n"/>
-      <c r="CV13" s="9" t="n"/>
+      <c r="CV13" s="12" t="n"/>
       <c r="CW13" s="9" t="n"/>
       <c r="CX13" s="11" t="inlineStr">
         <is>
@@ -1498,7 +1492,7 @@
       <c r="CY13" s="9" t="n"/>
       <c r="CZ13" s="9" t="n"/>
       <c r="DA13" s="9" t="n"/>
-      <c r="DB13" s="9" t="n"/>
+      <c r="DB13" s="12" t="n"/>
       <c r="DC13" s="9" t="n"/>
       <c r="DD13" s="11" t="inlineStr">
         <is>
@@ -1507,7 +1501,7 @@
       </c>
       <c r="DE13" s="9" t="n"/>
       <c r="DF13" s="9" t="n"/>
-      <c r="DG13" s="9" t="n"/>
+      <c r="DG13" s="12" t="n"/>
       <c r="DH13" s="9" t="n"/>
       <c r="DI13" s="11" t="inlineStr">
         <is>
@@ -1566,7 +1560,7 @@
       <c r="AU14" s="9" t="n"/>
       <c r="AV14" s="9" t="n"/>
       <c r="AW14" s="9" t="n"/>
-      <c r="AX14" s="10" t="n"/>
+      <c r="AX14" s="12" t="n"/>
       <c r="AY14" s="9" t="n"/>
       <c r="AZ14" s="9" t="n"/>
       <c r="BA14" s="11" t="inlineStr">
@@ -1575,30 +1569,30 @@
         </is>
       </c>
       <c r="BB14" s="9" t="n"/>
-      <c r="BC14" s="9" t="n"/>
+      <c r="BC14" s="12" t="n"/>
       <c r="BD14" s="9" t="n"/>
       <c r="BE14" s="9" t="n"/>
       <c r="BF14" s="9" t="n"/>
       <c r="BG14" s="9" t="n"/>
       <c r="BH14" s="9" t="n"/>
-      <c r="BI14" s="9" t="n"/>
+      <c r="BI14" s="12" t="n"/>
       <c r="BJ14" s="9" t="n"/>
       <c r="BK14" s="9" t="n"/>
       <c r="BL14" s="9" t="n"/>
       <c r="BM14" s="9" t="n"/>
-      <c r="BN14" s="17" t="n"/>
+      <c r="BN14" s="12" t="n"/>
       <c r="BO14" s="9" t="n"/>
       <c r="BP14" s="9" t="n"/>
       <c r="BQ14" s="9" t="n"/>
       <c r="BR14" s="9" t="n"/>
       <c r="BS14" s="9" t="n"/>
-      <c r="BT14" s="9" t="n"/>
+      <c r="BT14" s="12" t="n"/>
       <c r="BU14" s="9" t="n"/>
       <c r="BV14" s="9" t="n"/>
       <c r="BW14" s="9" t="n"/>
       <c r="BX14" s="9" t="n"/>
       <c r="BY14" s="9" t="n"/>
-      <c r="BZ14" s="9" t="n"/>
+      <c r="BZ14" s="12" t="n"/>
       <c r="CA14" s="9" t="n"/>
       <c r="CB14" s="9" t="n"/>
       <c r="CC14" s="9" t="n"/>
@@ -1609,7 +1603,7 @@
       <c r="CH14" s="9" t="n"/>
       <c r="CI14" s="9" t="n"/>
       <c r="CJ14" s="9" t="n"/>
-      <c r="CK14" s="9" t="n"/>
+      <c r="CK14" s="12" t="n"/>
       <c r="CL14" s="9" t="n"/>
       <c r="CM14" s="9" t="n"/>
       <c r="CN14" s="11" t="inlineStr">
@@ -1619,12 +1613,12 @@
       </c>
       <c r="CO14" s="9" t="n"/>
       <c r="CP14" s="9" t="n"/>
-      <c r="CQ14" s="9" t="n"/>
+      <c r="CQ14" s="12" t="n"/>
       <c r="CR14" s="9" t="n"/>
       <c r="CS14" s="9" t="n"/>
       <c r="CT14" s="9" t="n"/>
       <c r="CU14" s="9" t="n"/>
-      <c r="CV14" s="11" t="inlineStr">
+      <c r="CV14" s="8" t="inlineStr">
         <is>
           <t>▼配分特性等整理完了</t>
         </is>
@@ -1634,12 +1628,12 @@
       <c r="CY14" s="9" t="n"/>
       <c r="CZ14" s="9" t="n"/>
       <c r="DA14" s="9" t="n"/>
-      <c r="DB14" s="9" t="n"/>
+      <c r="DB14" s="12" t="n"/>
       <c r="DC14" s="9" t="n"/>
       <c r="DD14" s="9" t="n"/>
       <c r="DE14" s="9" t="n"/>
       <c r="DF14" s="9" t="n"/>
-      <c r="DG14" s="9" t="n"/>
+      <c r="DG14" s="12" t="n"/>
       <c r="DH14" s="9" t="n"/>
       <c r="DI14" s="9" t="n"/>
       <c r="DJ14" s="9" t="n"/>
@@ -1690,7 +1684,7 @@
       <c r="AU15" s="13" t="n"/>
       <c r="AV15" s="13" t="n"/>
       <c r="AW15" s="13" t="n"/>
-      <c r="AX15" s="18" t="n"/>
+      <c r="AX15" s="14" t="n"/>
       <c r="AY15" s="13" t="n"/>
       <c r="AZ15" s="13" t="n"/>
       <c r="BA15" s="13" t="n"/>
@@ -1701,24 +1695,24 @@
       <c r="BF15" s="13" t="n"/>
       <c r="BG15" s="13" t="n"/>
       <c r="BH15" s="13" t="n"/>
-      <c r="BI15" s="13" t="n"/>
+      <c r="BI15" s="14" t="n"/>
       <c r="BJ15" s="13" t="n"/>
       <c r="BK15" s="13" t="n"/>
       <c r="BL15" s="13" t="n"/>
       <c r="BM15" s="13" t="n"/>
-      <c r="BN15" s="19" t="n"/>
+      <c r="BN15" s="14" t="n"/>
       <c r="BO15" s="13" t="n"/>
       <c r="BP15" s="13" t="n"/>
       <c r="BQ15" s="13" t="n"/>
       <c r="BR15" s="13" t="n"/>
       <c r="BS15" s="13" t="n"/>
-      <c r="BT15" s="13" t="n"/>
+      <c r="BT15" s="14" t="n"/>
       <c r="BU15" s="13" t="n"/>
       <c r="BV15" s="13" t="n"/>
       <c r="BW15" s="13" t="n"/>
       <c r="BX15" s="13" t="n"/>
       <c r="BY15" s="13" t="n"/>
-      <c r="BZ15" s="13" t="n"/>
+      <c r="BZ15" s="14" t="n"/>
       <c r="CA15" s="13" t="n"/>
       <c r="CB15" s="13" t="n"/>
       <c r="CC15" s="13" t="n"/>
@@ -1729,7 +1723,7 @@
       <c r="CH15" s="13" t="n"/>
       <c r="CI15" s="13" t="n"/>
       <c r="CJ15" s="13" t="n"/>
-      <c r="CK15" s="13" t="n"/>
+      <c r="CK15" s="14" t="n"/>
       <c r="CL15" s="13" t="n"/>
       <c r="CM15" s="13" t="n"/>
       <c r="CN15" s="13" t="n"/>
@@ -1740,7 +1734,7 @@
       <c r="CS15" s="13" t="n"/>
       <c r="CT15" s="13" t="n"/>
       <c r="CU15" s="13" t="n"/>
-      <c r="CV15" s="13" t="n"/>
+      <c r="CV15" s="14" t="n"/>
       <c r="CW15" s="13" t="n"/>
       <c r="CX15" s="13" t="n"/>
       <c r="CY15" s="13" t="n"/>
@@ -1751,13 +1745,13 @@
       <c r="DD15" s="13" t="n"/>
       <c r="DE15" s="13" t="n"/>
       <c r="DF15" s="13" t="n"/>
-      <c r="DG15" s="13" t="n"/>
+      <c r="DG15" s="14" t="n"/>
       <c r="DH15" s="13" t="n"/>
       <c r="DI15" s="13" t="n"/>
       <c r="DJ15" s="13" t="n"/>
       <c r="DK15" s="13" t="n"/>
       <c r="DL15" s="13" t="n"/>
-      <c r="DM15" s="18" t="n"/>
+      <c r="DM15" s="17" t="n"/>
     </row>
     <row r="16" ht="11.34" customHeight="1">
       <c r="H16" s="8" t="inlineStr">
@@ -1810,7 +1804,7 @@
       <c r="AU16" s="9" t="n"/>
       <c r="AV16" s="9" t="n"/>
       <c r="AW16" s="9" t="n"/>
-      <c r="AX16" s="10" t="n"/>
+      <c r="AX16" s="12" t="n"/>
       <c r="AY16" s="11" t="inlineStr">
         <is>
           <t>△</t>
@@ -1819,7 +1813,7 @@
       <c r="AZ16" s="9" t="n"/>
       <c r="BA16" s="9" t="n"/>
       <c r="BB16" s="9" t="n"/>
-      <c r="BC16" s="11" t="inlineStr">
+      <c r="BC16" s="8" t="inlineStr">
         <is>
           <t>△</t>
         </is>
@@ -1829,12 +1823,12 @@
       <c r="BF16" s="9" t="n"/>
       <c r="BG16" s="9" t="n"/>
       <c r="BH16" s="9" t="n"/>
-      <c r="BI16" s="9" t="n"/>
+      <c r="BI16" s="12" t="n"/>
       <c r="BJ16" s="9" t="n"/>
       <c r="BK16" s="9" t="n"/>
       <c r="BL16" s="9" t="n"/>
       <c r="BM16" s="9" t="n"/>
-      <c r="BN16" s="17" t="n"/>
+      <c r="BN16" s="12" t="n"/>
       <c r="BO16" s="9" t="n"/>
       <c r="BP16" s="11" t="inlineStr">
         <is>
@@ -1844,13 +1838,13 @@
       <c r="BQ16" s="9" t="n"/>
       <c r="BR16" s="9" t="n"/>
       <c r="BS16" s="9" t="n"/>
-      <c r="BT16" s="9" t="n"/>
+      <c r="BT16" s="12" t="n"/>
       <c r="BU16" s="9" t="n"/>
       <c r="BV16" s="9" t="n"/>
       <c r="BW16" s="9" t="n"/>
       <c r="BX16" s="9" t="n"/>
       <c r="BY16" s="9" t="n"/>
-      <c r="BZ16" s="9" t="n"/>
+      <c r="BZ16" s="12" t="n"/>
       <c r="CA16" s="9" t="n"/>
       <c r="CB16" s="9" t="n"/>
       <c r="CC16" s="9" t="n"/>
@@ -1865,13 +1859,13 @@
         </is>
       </c>
       <c r="CJ16" s="9" t="n"/>
-      <c r="CK16" s="9" t="n"/>
+      <c r="CK16" s="12" t="n"/>
       <c r="CL16" s="9" t="n"/>
       <c r="CM16" s="9" t="n"/>
       <c r="CN16" s="9" t="n"/>
       <c r="CO16" s="9" t="n"/>
       <c r="CP16" s="9" t="n"/>
-      <c r="CQ16" s="9" t="n"/>
+      <c r="CQ16" s="12" t="n"/>
       <c r="CR16" s="9" t="n"/>
       <c r="CS16" s="9" t="n"/>
       <c r="CT16" s="11" t="inlineStr">
@@ -1880,7 +1874,7 @@
         </is>
       </c>
       <c r="CU16" s="9" t="n"/>
-      <c r="CV16" s="9" t="n"/>
+      <c r="CV16" s="12" t="n"/>
       <c r="CW16" s="9" t="n"/>
       <c r="CX16" s="11" t="inlineStr">
         <is>
@@ -1890,12 +1884,12 @@
       <c r="CY16" s="9" t="n"/>
       <c r="CZ16" s="9" t="n"/>
       <c r="DA16" s="9" t="n"/>
-      <c r="DB16" s="9" t="n"/>
+      <c r="DB16" s="12" t="n"/>
       <c r="DC16" s="9" t="n"/>
       <c r="DD16" s="9" t="n"/>
       <c r="DE16" s="9" t="n"/>
       <c r="DF16" s="9" t="n"/>
-      <c r="DG16" s="9" t="n"/>
+      <c r="DG16" s="12" t="n"/>
       <c r="DH16" s="9" t="n"/>
       <c r="DI16" s="9" t="n"/>
       <c r="DJ16" s="9" t="n"/>
@@ -1954,7 +1948,7 @@
       <c r="AU17" s="9" t="n"/>
       <c r="AV17" s="9" t="n"/>
       <c r="AW17" s="9" t="n"/>
-      <c r="AX17" s="10" t="n"/>
+      <c r="AX17" s="12" t="n"/>
       <c r="AY17" s="11" t="inlineStr">
         <is>
           <t>△</t>
@@ -1963,7 +1957,7 @@
       <c r="AZ17" s="9" t="n"/>
       <c r="BA17" s="9" t="n"/>
       <c r="BB17" s="9" t="n"/>
-      <c r="BC17" s="11" t="inlineStr">
+      <c r="BC17" s="8" t="inlineStr">
         <is>
           <t>△</t>
         </is>
@@ -1977,12 +1971,12 @@
         </is>
       </c>
       <c r="BH17" s="9" t="n"/>
-      <c r="BI17" s="9" t="n"/>
+      <c r="BI17" s="12" t="n"/>
       <c r="BJ17" s="9" t="n"/>
       <c r="BK17" s="9" t="n"/>
       <c r="BL17" s="9" t="n"/>
       <c r="BM17" s="9" t="n"/>
-      <c r="BN17" s="17" t="n"/>
+      <c r="BN17" s="12" t="n"/>
       <c r="BO17" s="9" t="n"/>
       <c r="BP17" s="9" t="n"/>
       <c r="BQ17" s="9" t="n"/>
@@ -1992,13 +1986,13 @@
         </is>
       </c>
       <c r="BS17" s="9" t="n"/>
-      <c r="BT17" s="9" t="n"/>
+      <c r="BT17" s="12" t="n"/>
       <c r="BU17" s="9" t="n"/>
       <c r="BV17" s="9" t="n"/>
       <c r="BW17" s="9" t="n"/>
       <c r="BX17" s="9" t="n"/>
       <c r="BY17" s="9" t="n"/>
-      <c r="BZ17" s="9" t="n"/>
+      <c r="BZ17" s="12" t="n"/>
       <c r="CA17" s="9" t="n"/>
       <c r="CB17" s="9" t="n"/>
       <c r="CC17" s="9" t="n"/>
@@ -2009,29 +2003,29 @@
       <c r="CH17" s="9" t="n"/>
       <c r="CI17" s="9" t="n"/>
       <c r="CJ17" s="9" t="n"/>
-      <c r="CK17" s="9" t="n"/>
+      <c r="CK17" s="12" t="n"/>
       <c r="CL17" s="9" t="n"/>
       <c r="CM17" s="9" t="n"/>
       <c r="CN17" s="9" t="n"/>
       <c r="CO17" s="9" t="n"/>
       <c r="CP17" s="9" t="n"/>
-      <c r="CQ17" s="9" t="n"/>
+      <c r="CQ17" s="12" t="n"/>
       <c r="CR17" s="9" t="n"/>
       <c r="CS17" s="9" t="n"/>
       <c r="CT17" s="9" t="n"/>
       <c r="CU17" s="9" t="n"/>
-      <c r="CV17" s="9" t="n"/>
+      <c r="CV17" s="12" t="n"/>
       <c r="CW17" s="9" t="n"/>
       <c r="CX17" s="9" t="n"/>
       <c r="CY17" s="9" t="n"/>
       <c r="CZ17" s="9" t="n"/>
       <c r="DA17" s="9" t="n"/>
-      <c r="DB17" s="9" t="n"/>
+      <c r="DB17" s="12" t="n"/>
       <c r="DC17" s="9" t="n"/>
       <c r="DD17" s="9" t="n"/>
       <c r="DE17" s="9" t="n"/>
       <c r="DF17" s="9" t="n"/>
-      <c r="DG17" s="9" t="n"/>
+      <c r="DG17" s="12" t="n"/>
       <c r="DH17" s="9" t="n"/>
       <c r="DI17" s="9" t="n"/>
       <c r="DJ17" s="9" t="n"/>
@@ -2098,35 +2092,35 @@
           <t>14</t>
         </is>
       </c>
-      <c r="AX18" s="18" t="n"/>
+      <c r="AX18" s="14" t="n"/>
       <c r="AY18" s="13" t="n"/>
       <c r="AZ18" s="13" t="n"/>
       <c r="BA18" s="13" t="n"/>
       <c r="BB18" s="13" t="n"/>
-      <c r="BC18" s="13" t="n"/>
+      <c r="BC18" s="14" t="n"/>
       <c r="BD18" s="13" t="n"/>
       <c r="BE18" s="13" t="n"/>
       <c r="BF18" s="13" t="n"/>
       <c r="BG18" s="13" t="n"/>
       <c r="BH18" s="13" t="n"/>
-      <c r="BI18" s="13" t="n"/>
+      <c r="BI18" s="14" t="n"/>
       <c r="BJ18" s="13" t="n"/>
       <c r="BK18" s="13" t="n"/>
       <c r="BL18" s="13" t="n"/>
       <c r="BM18" s="13" t="n"/>
-      <c r="BN18" s="19" t="n"/>
+      <c r="BN18" s="14" t="n"/>
       <c r="BO18" s="13" t="n"/>
       <c r="BP18" s="13" t="n"/>
       <c r="BQ18" s="13" t="n"/>
       <c r="BR18" s="13" t="n"/>
       <c r="BS18" s="13" t="n"/>
-      <c r="BT18" s="13" t="n"/>
+      <c r="BT18" s="14" t="n"/>
       <c r="BU18" s="13" t="n"/>
       <c r="BV18" s="13" t="n"/>
       <c r="BW18" s="13" t="n"/>
       <c r="BX18" s="13" t="n"/>
       <c r="BY18" s="13" t="n"/>
-      <c r="BZ18" s="13" t="n"/>
+      <c r="BZ18" s="14" t="n"/>
       <c r="CA18" s="13" t="n"/>
       <c r="CB18" s="13" t="n"/>
       <c r="CC18" s="13" t="n"/>
@@ -2137,35 +2131,35 @@
       <c r="CH18" s="13" t="n"/>
       <c r="CI18" s="13" t="n"/>
       <c r="CJ18" s="13" t="n"/>
-      <c r="CK18" s="13" t="n"/>
+      <c r="CK18" s="14" t="n"/>
       <c r="CL18" s="13" t="n"/>
       <c r="CM18" s="13" t="n"/>
       <c r="CN18" s="13" t="n"/>
       <c r="CO18" s="13" t="n"/>
       <c r="CP18" s="13" t="n"/>
-      <c r="CQ18" s="13" t="n"/>
+      <c r="CQ18" s="14" t="n"/>
       <c r="CR18" s="13" t="n"/>
       <c r="CS18" s="13" t="n"/>
       <c r="CT18" s="13" t="n"/>
       <c r="CU18" s="13" t="n"/>
-      <c r="CV18" s="13" t="n"/>
+      <c r="CV18" s="14" t="n"/>
       <c r="CW18" s="13" t="n"/>
       <c r="CX18" s="13" t="n"/>
       <c r="CY18" s="13" t="n"/>
       <c r="CZ18" s="13" t="n"/>
       <c r="DA18" s="13" t="n"/>
-      <c r="DB18" s="13" t="n"/>
+      <c r="DB18" s="14" t="n"/>
       <c r="DC18" s="13" t="n"/>
       <c r="DD18" s="13" t="n"/>
       <c r="DE18" s="13" t="n"/>
       <c r="DF18" s="13" t="n"/>
-      <c r="DG18" s="13" t="n"/>
+      <c r="DG18" s="14" t="n"/>
       <c r="DH18" s="13" t="n"/>
       <c r="DI18" s="13" t="n"/>
       <c r="DJ18" s="13" t="n"/>
       <c r="DK18" s="13" t="n"/>
       <c r="DL18" s="13" t="n"/>
-      <c r="DM18" s="18" t="n"/>
+      <c r="DM18" s="17" t="n"/>
     </row>
     <row r="19" ht="11.34" customHeight="1">
       <c r="H19" s="16" t="inlineStr">
@@ -2234,35 +2228,35 @@
           <t>17</t>
         </is>
       </c>
-      <c r="AX19" s="10" t="n"/>
+      <c r="AX19" s="12" t="n"/>
       <c r="AY19" s="9" t="n"/>
       <c r="AZ19" s="9" t="n"/>
       <c r="BA19" s="9" t="n"/>
       <c r="BB19" s="9" t="n"/>
-      <c r="BC19" s="9" t="n"/>
+      <c r="BC19" s="12" t="n"/>
       <c r="BD19" s="13" t="n"/>
       <c r="BE19" s="13" t="n"/>
       <c r="BF19" s="13" t="n"/>
       <c r="BG19" s="13" t="n"/>
       <c r="BH19" s="13" t="n"/>
-      <c r="BI19" s="13" t="n"/>
+      <c r="BI19" s="14" t="n"/>
       <c r="BJ19" s="13" t="n"/>
       <c r="BK19" s="13" t="n"/>
       <c r="BL19" s="13" t="n"/>
       <c r="BM19" s="13" t="n"/>
-      <c r="BN19" s="19" t="n"/>
+      <c r="BN19" s="14" t="n"/>
       <c r="BO19" s="13" t="n"/>
       <c r="BP19" s="13" t="n"/>
       <c r="BQ19" s="13" t="n"/>
       <c r="BR19" s="13" t="n"/>
       <c r="BS19" s="13" t="n"/>
-      <c r="BT19" s="13" t="n"/>
+      <c r="BT19" s="14" t="n"/>
       <c r="BU19" s="13" t="n"/>
       <c r="BV19" s="13" t="n"/>
       <c r="BW19" s="13" t="n"/>
       <c r="BX19" s="13" t="n"/>
       <c r="BY19" s="13" t="n"/>
-      <c r="BZ19" s="13" t="n"/>
+      <c r="BZ19" s="14" t="n"/>
       <c r="CA19" s="13" t="n"/>
       <c r="CB19" s="13" t="n"/>
       <c r="CC19" s="13" t="n"/>
@@ -2277,35 +2271,35 @@
       <c r="CH19" s="9" t="n"/>
       <c r="CI19" s="9" t="n"/>
       <c r="CJ19" s="9" t="n"/>
-      <c r="CK19" s="9" t="n"/>
+      <c r="CK19" s="12" t="n"/>
       <c r="CL19" s="9" t="n"/>
       <c r="CM19" s="9" t="n"/>
       <c r="CN19" s="9" t="n"/>
       <c r="CO19" s="9" t="n"/>
       <c r="CP19" s="9" t="n"/>
-      <c r="CQ19" s="9" t="n"/>
+      <c r="CQ19" s="12" t="n"/>
       <c r="CR19" s="9" t="n"/>
       <c r="CS19" s="13" t="n"/>
       <c r="CT19" s="13" t="n"/>
       <c r="CU19" s="13" t="n"/>
-      <c r="CV19" s="13" t="n"/>
+      <c r="CV19" s="14" t="n"/>
       <c r="CW19" s="13" t="n"/>
       <c r="CX19" s="13" t="n"/>
       <c r="CY19" s="13" t="n"/>
       <c r="CZ19" s="13" t="n"/>
       <c r="DA19" s="13" t="n"/>
-      <c r="DB19" s="13" t="n"/>
+      <c r="DB19" s="14" t="n"/>
       <c r="DC19" s="13" t="n"/>
       <c r="DD19" s="13" t="n"/>
       <c r="DE19" s="13" t="n"/>
       <c r="DF19" s="13" t="n"/>
-      <c r="DG19" s="13" t="n"/>
+      <c r="DG19" s="14" t="n"/>
       <c r="DH19" s="13" t="n"/>
       <c r="DI19" s="13" t="n"/>
       <c r="DJ19" s="13" t="n"/>
       <c r="DK19" s="13" t="n"/>
       <c r="DL19" s="13" t="n"/>
-      <c r="DM19" s="18" t="n"/>
+      <c r="DM19" s="17" t="n"/>
     </row>
     <row r="20" ht="11.34" customHeight="1">
       <c r="H20" s="14" t="n"/>
@@ -2350,42 +2344,42 @@
       <c r="AU20" s="13" t="n"/>
       <c r="AV20" s="13" t="n"/>
       <c r="AW20" s="13" t="n"/>
-      <c r="AX20" s="18" t="n"/>
+      <c r="AX20" s="14" t="n"/>
       <c r="AY20" s="13" t="n"/>
       <c r="AZ20" s="13" t="n"/>
       <c r="BA20" s="13" t="n"/>
       <c r="BB20" s="13" t="n"/>
-      <c r="BC20" s="13" t="n"/>
+      <c r="BC20" s="14" t="n"/>
       <c r="BD20" s="13" t="n"/>
       <c r="BE20" s="13" t="n"/>
       <c r="BF20" s="13" t="n"/>
       <c r="BG20" s="13" t="n"/>
       <c r="BH20" s="13" t="n"/>
-      <c r="BI20" s="13" t="n"/>
+      <c r="BI20" s="14" t="n"/>
       <c r="BJ20" s="13" t="n"/>
       <c r="BK20" s="13" t="n"/>
       <c r="BL20" s="13" t="n"/>
       <c r="BM20" s="13" t="n"/>
-      <c r="BN20" s="19" t="n"/>
+      <c r="BN20" s="14" t="n"/>
       <c r="BO20" s="13" t="n"/>
       <c r="BP20" s="13" t="n"/>
       <c r="BQ20" s="13" t="n"/>
       <c r="BR20" s="13" t="n"/>
       <c r="BS20" s="13" t="n"/>
-      <c r="BT20" s="13" t="n"/>
+      <c r="BT20" s="14" t="n"/>
       <c r="BU20" s="13" t="n"/>
       <c r="BV20" s="13" t="n"/>
       <c r="BW20" s="13" t="n"/>
       <c r="BX20" s="13" t="n"/>
       <c r="BY20" s="13" t="n"/>
-      <c r="BZ20" s="13" t="n"/>
+      <c r="BZ20" s="14" t="n"/>
       <c r="CA20" s="13" t="n"/>
       <c r="CB20" s="13" t="n"/>
       <c r="CC20" s="13" t="n"/>
       <c r="CD20" s="13" t="n"/>
       <c r="CE20" s="13" t="n"/>
       <c r="CF20" s="13" t="n"/>
-      <c r="CG20" s="20" t="inlineStr">
+      <c r="CG20" s="15" t="inlineStr">
         <is>
           <t>書式設定」から色を設定することが</t>
         </is>
@@ -2393,35 +2387,35 @@
       <c r="CH20" s="13" t="n"/>
       <c r="CI20" s="13" t="n"/>
       <c r="CJ20" s="13" t="n"/>
-      <c r="CK20" s="13" t="n"/>
+      <c r="CK20" s="14" t="n"/>
       <c r="CL20" s="13" t="n"/>
       <c r="CM20" s="13" t="n"/>
       <c r="CN20" s="13" t="n"/>
       <c r="CO20" s="13" t="n"/>
       <c r="CP20" s="13" t="n"/>
-      <c r="CQ20" s="13" t="n"/>
+      <c r="CQ20" s="14" t="n"/>
       <c r="CR20" s="13" t="n"/>
       <c r="CS20" s="13" t="n"/>
       <c r="CT20" s="13" t="n"/>
       <c r="CU20" s="13" t="n"/>
-      <c r="CV20" s="13" t="n"/>
+      <c r="CV20" s="14" t="n"/>
       <c r="CW20" s="13" t="n"/>
       <c r="CX20" s="13" t="n"/>
       <c r="CY20" s="13" t="n"/>
       <c r="CZ20" s="13" t="n"/>
       <c r="DA20" s="13" t="n"/>
-      <c r="DB20" s="13" t="n"/>
+      <c r="DB20" s="14" t="n"/>
       <c r="DC20" s="13" t="n"/>
       <c r="DD20" s="13" t="n"/>
       <c r="DE20" s="13" t="n"/>
       <c r="DF20" s="13" t="n"/>
-      <c r="DG20" s="13" t="n"/>
+      <c r="DG20" s="14" t="n"/>
       <c r="DH20" s="13" t="n"/>
       <c r="DI20" s="13" t="n"/>
       <c r="DJ20" s="13" t="n"/>
       <c r="DK20" s="13" t="n"/>
       <c r="DL20" s="13" t="n"/>
-      <c r="DM20" s="18" t="n"/>
+      <c r="DM20" s="17" t="n"/>
     </row>
     <row r="21" ht="11.34" customHeight="1">
       <c r="H21" s="16" t="inlineStr">
@@ -2471,7 +2465,7 @@
       <c r="AJ21" s="12" t="n"/>
       <c r="AK21" s="11" t="inlineStr">
         <is>
-          <t>実績</t>
+          <t>計画</t>
         </is>
       </c>
       <c r="AL21" s="9" t="n"/>
@@ -2490,35 +2484,35 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AX21" s="18" t="n"/>
+      <c r="AX21" s="14" t="n"/>
       <c r="AY21" s="13" t="n"/>
       <c r="AZ21" s="13" t="n"/>
       <c r="BA21" s="13" t="n"/>
       <c r="BB21" s="13" t="n"/>
-      <c r="BC21" s="9" t="n"/>
+      <c r="BC21" s="12" t="n"/>
       <c r="BD21" s="9" t="n"/>
       <c r="BE21" s="9" t="n"/>
       <c r="BF21" s="9" t="n"/>
       <c r="BG21" s="9" t="n"/>
       <c r="BH21" s="13" t="n"/>
-      <c r="BI21" s="13" t="n"/>
+      <c r="BI21" s="14" t="n"/>
       <c r="BJ21" s="13" t="n"/>
       <c r="BK21" s="9" t="n"/>
       <c r="BL21" s="9" t="n"/>
       <c r="BM21" s="9" t="n"/>
-      <c r="BN21" s="17" t="n"/>
+      <c r="BN21" s="12" t="n"/>
       <c r="BO21" s="9" t="n"/>
       <c r="BP21" s="9" t="n"/>
       <c r="BQ21" s="10" t="n"/>
       <c r="BR21" s="13" t="n"/>
       <c r="BS21" s="13" t="n"/>
-      <c r="BT21" s="13" t="n"/>
+      <c r="BT21" s="14" t="n"/>
       <c r="BU21" s="13" t="n"/>
       <c r="BV21" s="9" t="n"/>
       <c r="BW21" s="9" t="n"/>
       <c r="BX21" s="9" t="n"/>
       <c r="BY21" s="9" t="n"/>
-      <c r="BZ21" s="9" t="n"/>
+      <c r="BZ21" s="12" t="n"/>
       <c r="CA21" s="13" t="n"/>
       <c r="CB21" s="13" t="n"/>
       <c r="CC21" s="13" t="n"/>
@@ -2529,35 +2523,35 @@
       <c r="CH21" s="9" t="n"/>
       <c r="CI21" s="9" t="n"/>
       <c r="CJ21" s="9" t="n"/>
-      <c r="CK21" s="9" t="n"/>
+      <c r="CK21" s="12" t="n"/>
       <c r="CL21" s="9" t="n"/>
       <c r="CM21" s="9" t="n"/>
       <c r="CN21" s="9" t="n"/>
       <c r="CO21" s="9" t="n"/>
       <c r="CP21" s="9" t="n"/>
-      <c r="CQ21" s="9" t="n"/>
+      <c r="CQ21" s="12" t="n"/>
       <c r="CR21" s="9" t="n"/>
       <c r="CS21" s="13" t="n"/>
       <c r="CT21" s="13" t="n"/>
       <c r="CU21" s="13" t="n"/>
-      <c r="CV21" s="13" t="n"/>
+      <c r="CV21" s="14" t="n"/>
       <c r="CW21" s="13" t="n"/>
       <c r="CX21" s="13" t="n"/>
       <c r="CY21" s="13" t="n"/>
       <c r="CZ21" s="13" t="n"/>
       <c r="DA21" s="13" t="n"/>
-      <c r="DB21" s="13" t="n"/>
+      <c r="DB21" s="14" t="n"/>
       <c r="DC21" s="13" t="n"/>
       <c r="DD21" s="13" t="n"/>
       <c r="DE21" s="13" t="n"/>
       <c r="DF21" s="13" t="n"/>
-      <c r="DG21" s="13" t="n"/>
+      <c r="DG21" s="14" t="n"/>
       <c r="DH21" s="13" t="n"/>
       <c r="DI21" s="13" t="n"/>
       <c r="DJ21" s="13" t="n"/>
       <c r="DK21" s="13" t="n"/>
       <c r="DL21" s="13" t="n"/>
-      <c r="DM21" s="18" t="n"/>
+      <c r="DM21" s="17" t="n"/>
     </row>
     <row r="22" ht="11.34" customHeight="1">
       <c r="H22" s="14" t="n"/>
@@ -2577,7 +2571,7 @@
       <c r="V22" s="13" t="n"/>
       <c r="W22" s="13" t="n"/>
       <c r="X22" s="13" t="n"/>
-      <c r="Y22" s="21" t="inlineStr">
+      <c r="Y22" s="18" t="inlineStr">
         <is>
           <t>応できるようテキスト、罫線</t>
         </is>
@@ -2606,35 +2600,35 @@
       <c r="AU22" s="13" t="n"/>
       <c r="AV22" s="13" t="n"/>
       <c r="AW22" s="13" t="n"/>
-      <c r="AX22" s="18" t="n"/>
+      <c r="AX22" s="14" t="n"/>
       <c r="AY22" s="13" t="n"/>
       <c r="AZ22" s="13" t="n"/>
       <c r="BA22" s="13" t="n"/>
       <c r="BB22" s="13" t="n"/>
-      <c r="BC22" s="13" t="n"/>
+      <c r="BC22" s="14" t="n"/>
       <c r="BD22" s="13" t="n"/>
       <c r="BE22" s="13" t="n"/>
       <c r="BF22" s="13" t="n"/>
       <c r="BG22" s="13" t="n"/>
       <c r="BH22" s="13" t="n"/>
-      <c r="BI22" s="13" t="n"/>
+      <c r="BI22" s="14" t="n"/>
       <c r="BJ22" s="13" t="n"/>
       <c r="BK22" s="13" t="n"/>
       <c r="BL22" s="13" t="n"/>
       <c r="BM22" s="13" t="n"/>
-      <c r="BN22" s="19" t="n"/>
+      <c r="BN22" s="14" t="n"/>
       <c r="BO22" s="13" t="n"/>
       <c r="BP22" s="13" t="n"/>
-      <c r="BQ22" s="18" t="n"/>
+      <c r="BQ22" s="17" t="n"/>
       <c r="BR22" s="13" t="n"/>
       <c r="BS22" s="13" t="n"/>
-      <c r="BT22" s="13" t="n"/>
+      <c r="BT22" s="14" t="n"/>
       <c r="BU22" s="13" t="n"/>
       <c r="BV22" s="13" t="n"/>
       <c r="BW22" s="13" t="n"/>
       <c r="BX22" s="13" t="n"/>
       <c r="BY22" s="13" t="n"/>
-      <c r="BZ22" s="13" t="n"/>
+      <c r="BZ22" s="14" t="n"/>
       <c r="CA22" s="13" t="n"/>
       <c r="CB22" s="13" t="n"/>
       <c r="CC22" s="13" t="n"/>
@@ -2645,35 +2639,35 @@
       <c r="CH22" s="13" t="n"/>
       <c r="CI22" s="13" t="n"/>
       <c r="CJ22" s="13" t="n"/>
-      <c r="CK22" s="13" t="n"/>
+      <c r="CK22" s="14" t="n"/>
       <c r="CL22" s="13" t="n"/>
       <c r="CM22" s="13" t="n"/>
       <c r="CN22" s="13" t="n"/>
       <c r="CO22" s="13" t="n"/>
       <c r="CP22" s="13" t="n"/>
-      <c r="CQ22" s="13" t="n"/>
+      <c r="CQ22" s="14" t="n"/>
       <c r="CR22" s="13" t="n"/>
       <c r="CS22" s="13" t="n"/>
       <c r="CT22" s="13" t="n"/>
       <c r="CU22" s="13" t="n"/>
-      <c r="CV22" s="13" t="n"/>
+      <c r="CV22" s="14" t="n"/>
       <c r="CW22" s="13" t="n"/>
       <c r="CX22" s="13" t="n"/>
       <c r="CY22" s="13" t="n"/>
       <c r="CZ22" s="13" t="n"/>
       <c r="DA22" s="13" t="n"/>
-      <c r="DB22" s="13" t="n"/>
+      <c r="DB22" s="14" t="n"/>
       <c r="DC22" s="13" t="n"/>
       <c r="DD22" s="13" t="n"/>
       <c r="DE22" s="13" t="n"/>
       <c r="DF22" s="13" t="n"/>
-      <c r="DG22" s="13" t="n"/>
+      <c r="DG22" s="14" t="n"/>
       <c r="DH22" s="13" t="n"/>
       <c r="DI22" s="13" t="n"/>
       <c r="DJ22" s="13" t="n"/>
       <c r="DK22" s="13" t="n"/>
       <c r="DL22" s="13" t="n"/>
-      <c r="DM22" s="18" t="n"/>
+      <c r="DM22" s="17" t="n"/>
     </row>
     <row r="23" ht="11.34" customHeight="1">
       <c r="H23" s="14" t="n"/>
@@ -2697,7 +2691,7 @@
       <c r="V23" s="9" t="n"/>
       <c r="W23" s="9" t="n"/>
       <c r="X23" s="9" t="n"/>
-      <c r="Y23" s="22" t="inlineStr">
+      <c r="Y23" s="19" t="inlineStr">
         <is>
           <t>等の編集が可能</t>
         </is>
@@ -2709,7 +2703,7 @@
       <c r="AD23" s="9" t="n"/>
       <c r="AE23" s="9" t="n"/>
       <c r="AF23" s="9" t="n"/>
-      <c r="AG23" s="23" t="inlineStr">
+      <c r="AG23" s="20" t="inlineStr">
         <is>
           <t>実施中</t>
         </is>
@@ -2746,35 +2740,35 @@
           <t>110</t>
         </is>
       </c>
-      <c r="AX23" s="10" t="n"/>
+      <c r="AX23" s="12" t="n"/>
       <c r="AY23" s="9" t="n"/>
       <c r="AZ23" s="9" t="n"/>
       <c r="BA23" s="9" t="n"/>
       <c r="BB23" s="9" t="n"/>
-      <c r="BC23" s="9" t="n"/>
+      <c r="BC23" s="12" t="n"/>
       <c r="BD23" s="9" t="n"/>
       <c r="BE23" s="9" t="n"/>
       <c r="BF23" s="9" t="n"/>
       <c r="BG23" s="9" t="n"/>
       <c r="BH23" s="9" t="n"/>
-      <c r="BI23" s="9" t="n"/>
+      <c r="BI23" s="12" t="n"/>
       <c r="BJ23" s="9" t="n"/>
       <c r="BK23" s="9" t="n"/>
       <c r="BL23" s="9" t="n"/>
       <c r="BM23" s="9" t="n"/>
-      <c r="BN23" s="17" t="n"/>
+      <c r="BN23" s="12" t="n"/>
       <c r="BO23" s="9" t="n"/>
       <c r="BP23" s="9" t="n"/>
       <c r="BQ23" s="10" t="n"/>
       <c r="BR23" s="9" t="n"/>
       <c r="BS23" s="9" t="n"/>
-      <c r="BT23" s="9" t="n"/>
+      <c r="BT23" s="12" t="n"/>
       <c r="BU23" s="9" t="n"/>
       <c r="BV23" s="9" t="n"/>
       <c r="BW23" s="9" t="n"/>
       <c r="BX23" s="9" t="n"/>
       <c r="BY23" s="9" t="n"/>
-      <c r="BZ23" s="9" t="n"/>
+      <c r="BZ23" s="12" t="n"/>
       <c r="CA23" s="9" t="n"/>
       <c r="CB23" s="9" t="n"/>
       <c r="CC23" s="9" t="n"/>
@@ -2785,29 +2779,29 @@
       <c r="CH23" s="9" t="n"/>
       <c r="CI23" s="9" t="n"/>
       <c r="CJ23" s="9" t="n"/>
-      <c r="CK23" s="9" t="n"/>
+      <c r="CK23" s="12" t="n"/>
       <c r="CL23" s="9" t="n"/>
       <c r="CM23" s="9" t="n"/>
       <c r="CN23" s="9" t="n"/>
       <c r="CO23" s="9" t="n"/>
       <c r="CP23" s="9" t="n"/>
-      <c r="CQ23" s="9" t="n"/>
+      <c r="CQ23" s="12" t="n"/>
       <c r="CR23" s="9" t="n"/>
       <c r="CS23" s="9" t="n"/>
       <c r="CT23" s="9" t="n"/>
       <c r="CU23" s="9" t="n"/>
-      <c r="CV23" s="9" t="n"/>
+      <c r="CV23" s="12" t="n"/>
       <c r="CW23" s="9" t="n"/>
       <c r="CX23" s="9" t="n"/>
       <c r="CY23" s="9" t="n"/>
       <c r="CZ23" s="9" t="n"/>
       <c r="DA23" s="9" t="n"/>
-      <c r="DB23" s="9" t="n"/>
+      <c r="DB23" s="12" t="n"/>
       <c r="DC23" s="9" t="n"/>
       <c r="DD23" s="9" t="n"/>
       <c r="DE23" s="9" t="n"/>
       <c r="DF23" s="9" t="n"/>
-      <c r="DG23" s="9" t="n"/>
+      <c r="DG23" s="12" t="n"/>
       <c r="DH23" s="9" t="n"/>
       <c r="DI23" s="9" t="n"/>
       <c r="DJ23" s="9" t="n"/>
@@ -2866,35 +2860,35 @@
       <c r="AU24" s="13" t="n"/>
       <c r="AV24" s="13" t="n"/>
       <c r="AW24" s="13" t="n"/>
-      <c r="AX24" s="18" t="n"/>
+      <c r="AX24" s="14" t="n"/>
       <c r="AY24" s="13" t="n"/>
       <c r="AZ24" s="13" t="n"/>
       <c r="BA24" s="13" t="n"/>
       <c r="BB24" s="13" t="n"/>
-      <c r="BC24" s="13" t="n"/>
+      <c r="BC24" s="14" t="n"/>
       <c r="BD24" s="13" t="n"/>
       <c r="BE24" s="13" t="n"/>
       <c r="BF24" s="13" t="n"/>
       <c r="BG24" s="13" t="n"/>
       <c r="BH24" s="13" t="n"/>
-      <c r="BI24" s="13" t="n"/>
+      <c r="BI24" s="14" t="n"/>
       <c r="BJ24" s="13" t="n"/>
       <c r="BK24" s="13" t="n"/>
       <c r="BL24" s="13" t="n"/>
       <c r="BM24" s="13" t="n"/>
-      <c r="BN24" s="19" t="n"/>
+      <c r="BN24" s="14" t="n"/>
       <c r="BO24" s="13" t="n"/>
       <c r="BP24" s="13" t="n"/>
       <c r="BQ24" s="13" t="n"/>
       <c r="BR24" s="13" t="n"/>
       <c r="BS24" s="13" t="n"/>
-      <c r="BT24" s="13" t="n"/>
+      <c r="BT24" s="14" t="n"/>
       <c r="BU24" s="13" t="n"/>
       <c r="BV24" s="13" t="n"/>
       <c r="BW24" s="13" t="n"/>
       <c r="BX24" s="13" t="n"/>
       <c r="BY24" s="13" t="n"/>
-      <c r="BZ24" s="13" t="n"/>
+      <c r="BZ24" s="14" t="n"/>
       <c r="CA24" s="13" t="n"/>
       <c r="CB24" s="13" t="n"/>
       <c r="CC24" s="13" t="n"/>
@@ -2905,35 +2899,35 @@
       <c r="CH24" s="13" t="n"/>
       <c r="CI24" s="13" t="n"/>
       <c r="CJ24" s="13" t="n"/>
-      <c r="CK24" s="13" t="n"/>
+      <c r="CK24" s="14" t="n"/>
       <c r="CL24" s="13" t="n"/>
       <c r="CM24" s="13" t="n"/>
       <c r="CN24" s="13" t="n"/>
       <c r="CO24" s="13" t="n"/>
       <c r="CP24" s="13" t="n"/>
-      <c r="CQ24" s="13" t="n"/>
+      <c r="CQ24" s="14" t="n"/>
       <c r="CR24" s="13" t="n"/>
       <c r="CS24" s="13" t="n"/>
       <c r="CT24" s="13" t="n"/>
       <c r="CU24" s="13" t="n"/>
-      <c r="CV24" s="13" t="n"/>
+      <c r="CV24" s="14" t="n"/>
       <c r="CW24" s="13" t="n"/>
       <c r="CX24" s="13" t="n"/>
       <c r="CY24" s="13" t="n"/>
       <c r="CZ24" s="13" t="n"/>
       <c r="DA24" s="13" t="n"/>
-      <c r="DB24" s="13" t="n"/>
+      <c r="DB24" s="14" t="n"/>
       <c r="DC24" s="13" t="n"/>
       <c r="DD24" s="13" t="n"/>
       <c r="DE24" s="13" t="n"/>
       <c r="DF24" s="13" t="n"/>
-      <c r="DG24" s="13" t="n"/>
+      <c r="DG24" s="14" t="n"/>
       <c r="DH24" s="13" t="n"/>
       <c r="DI24" s="13" t="n"/>
       <c r="DJ24" s="13" t="n"/>
       <c r="DK24" s="13" t="n"/>
       <c r="DL24" s="13" t="n"/>
-      <c r="DM24" s="18" t="n"/>
+      <c r="DM24" s="17" t="n"/>
     </row>
     <row r="25" ht="11.34" customHeight="1">
       <c r="H25" s="8" t="inlineStr">
@@ -3006,23 +3000,23 @@
           <t>28</t>
         </is>
       </c>
-      <c r="AX25" s="10" t="n"/>
+      <c r="AX25" s="12" t="n"/>
       <c r="AY25" s="9" t="n"/>
       <c r="AZ25" s="9" t="n"/>
       <c r="BA25" s="9" t="n"/>
       <c r="BB25" s="9" t="n"/>
-      <c r="BC25" s="9" t="n"/>
+      <c r="BC25" s="12" t="n"/>
       <c r="BD25" s="9" t="n"/>
       <c r="BE25" s="9" t="n"/>
       <c r="BF25" s="9" t="n"/>
       <c r="BG25" s="9" t="n"/>
       <c r="BH25" s="9" t="n"/>
-      <c r="BI25" s="9" t="n"/>
+      <c r="BI25" s="12" t="n"/>
       <c r="BJ25" s="9" t="n"/>
       <c r="BK25" s="9" t="n"/>
       <c r="BL25" s="9" t="n"/>
       <c r="BM25" s="9" t="n"/>
-      <c r="BN25" s="24" t="inlineStr">
+      <c r="BN25" s="8" t="inlineStr">
         <is>
           <t>バーチャートは入力した着手日、完了日をもとにマクロを使用して表示</t>
         </is>
@@ -3032,13 +3026,13 @@
       <c r="BQ25" s="9" t="n"/>
       <c r="BR25" s="9" t="n"/>
       <c r="BS25" s="9" t="n"/>
-      <c r="BT25" s="9" t="n"/>
+      <c r="BT25" s="12" t="n"/>
       <c r="BU25" s="9" t="n"/>
       <c r="BV25" s="9" t="n"/>
       <c r="BW25" s="9" t="n"/>
       <c r="BX25" s="9" t="n"/>
       <c r="BY25" s="9" t="n"/>
-      <c r="BZ25" s="9" t="n"/>
+      <c r="BZ25" s="12" t="n"/>
       <c r="CA25" s="9" t="n"/>
       <c r="CB25" s="9" t="n"/>
       <c r="CC25" s="9" t="n"/>
@@ -3049,29 +3043,29 @@
       <c r="CH25" s="9" t="n"/>
       <c r="CI25" s="9" t="n"/>
       <c r="CJ25" s="9" t="n"/>
-      <c r="CK25" s="9" t="n"/>
+      <c r="CK25" s="12" t="n"/>
       <c r="CL25" s="9" t="n"/>
       <c r="CM25" s="9" t="n"/>
       <c r="CN25" s="9" t="n"/>
       <c r="CO25" s="9" t="n"/>
       <c r="CP25" s="9" t="n"/>
-      <c r="CQ25" s="9" t="n"/>
+      <c r="CQ25" s="12" t="n"/>
       <c r="CR25" s="9" t="n"/>
       <c r="CS25" s="9" t="n"/>
       <c r="CT25" s="9" t="n"/>
       <c r="CU25" s="9" t="n"/>
-      <c r="CV25" s="9" t="n"/>
+      <c r="CV25" s="12" t="n"/>
       <c r="CW25" s="9" t="n"/>
       <c r="CX25" s="9" t="n"/>
       <c r="CY25" s="9" t="n"/>
       <c r="CZ25" s="9" t="n"/>
       <c r="DA25" s="9" t="n"/>
-      <c r="DB25" s="9" t="n"/>
+      <c r="DB25" s="12" t="n"/>
       <c r="DC25" s="9" t="n"/>
       <c r="DD25" s="9" t="n"/>
       <c r="DE25" s="9" t="n"/>
       <c r="DF25" s="9" t="n"/>
-      <c r="DG25" s="9" t="n"/>
+      <c r="DG25" s="12" t="n"/>
       <c r="DH25" s="9" t="n"/>
       <c r="DI25" s="9" t="n"/>
       <c r="DJ25" s="9" t="n"/>
@@ -3138,35 +3132,35 @@
           <t>28</t>
         </is>
       </c>
-      <c r="AX26" s="18" t="n"/>
+      <c r="AX26" s="14" t="n"/>
       <c r="AY26" s="13" t="n"/>
       <c r="AZ26" s="13" t="n"/>
       <c r="BA26" s="13" t="n"/>
       <c r="BB26" s="13" t="n"/>
-      <c r="BC26" s="13" t="n"/>
+      <c r="BC26" s="14" t="n"/>
       <c r="BD26" s="13" t="n"/>
       <c r="BE26" s="13" t="n"/>
       <c r="BF26" s="13" t="n"/>
       <c r="BG26" s="13" t="n"/>
       <c r="BH26" s="13" t="n"/>
-      <c r="BI26" s="13" t="n"/>
+      <c r="BI26" s="14" t="n"/>
       <c r="BJ26" s="13" t="n"/>
       <c r="BK26" s="13" t="n"/>
       <c r="BL26" s="13" t="n"/>
       <c r="BM26" s="13" t="n"/>
-      <c r="BN26" s="19" t="n"/>
+      <c r="BN26" s="14" t="n"/>
       <c r="BO26" s="13" t="n"/>
       <c r="BP26" s="13" t="n"/>
       <c r="BQ26" s="13" t="n"/>
       <c r="BR26" s="13" t="n"/>
       <c r="BS26" s="13" t="n"/>
-      <c r="BT26" s="13" t="n"/>
+      <c r="BT26" s="14" t="n"/>
       <c r="BU26" s="13" t="n"/>
       <c r="BV26" s="13" t="n"/>
       <c r="BW26" s="13" t="n"/>
       <c r="BX26" s="13" t="n"/>
       <c r="BY26" s="13" t="n"/>
-      <c r="BZ26" s="13" t="n"/>
+      <c r="BZ26" s="14" t="n"/>
       <c r="CA26" s="13" t="n"/>
       <c r="CB26" s="13" t="n"/>
       <c r="CC26" s="13" t="n"/>
@@ -3177,35 +3171,35 @@
       <c r="CH26" s="13" t="n"/>
       <c r="CI26" s="13" t="n"/>
       <c r="CJ26" s="13" t="n"/>
-      <c r="CK26" s="13" t="n"/>
+      <c r="CK26" s="14" t="n"/>
       <c r="CL26" s="13" t="n"/>
       <c r="CM26" s="13" t="n"/>
       <c r="CN26" s="13" t="n"/>
       <c r="CO26" s="13" t="n"/>
       <c r="CP26" s="13" t="n"/>
-      <c r="CQ26" s="13" t="n"/>
+      <c r="CQ26" s="14" t="n"/>
       <c r="CR26" s="13" t="n"/>
       <c r="CS26" s="13" t="n"/>
       <c r="CT26" s="13" t="n"/>
       <c r="CU26" s="13" t="n"/>
-      <c r="CV26" s="13" t="n"/>
+      <c r="CV26" s="14" t="n"/>
       <c r="CW26" s="13" t="n"/>
       <c r="CX26" s="13" t="n"/>
       <c r="CY26" s="13" t="n"/>
       <c r="CZ26" s="13" t="n"/>
       <c r="DA26" s="13" t="n"/>
-      <c r="DB26" s="13" t="n"/>
+      <c r="DB26" s="14" t="n"/>
       <c r="DC26" s="13" t="n"/>
       <c r="DD26" s="13" t="n"/>
       <c r="DE26" s="13" t="n"/>
       <c r="DF26" s="13" t="n"/>
-      <c r="DG26" s="13" t="n"/>
+      <c r="DG26" s="14" t="n"/>
       <c r="DH26" s="13" t="n"/>
       <c r="DI26" s="13" t="n"/>
       <c r="DJ26" s="13" t="n"/>
       <c r="DK26" s="13" t="n"/>
       <c r="DL26" s="13" t="n"/>
-      <c r="DM26" s="18" t="n"/>
+      <c r="DM26" s="17" t="n"/>
     </row>
     <row r="27" ht="11.34" customHeight="1">
       <c r="H27" s="14" t="n"/>
@@ -3274,23 +3268,23 @@
           <t>28</t>
         </is>
       </c>
-      <c r="AX27" s="10" t="n"/>
+      <c r="AX27" s="12" t="n"/>
       <c r="AY27" s="9" t="n"/>
       <c r="AZ27" s="9" t="n"/>
       <c r="BA27" s="9" t="n"/>
       <c r="BB27" s="9" t="n"/>
-      <c r="BC27" s="9" t="n"/>
+      <c r="BC27" s="12" t="n"/>
       <c r="BD27" s="9" t="n"/>
       <c r="BE27" s="9" t="n"/>
       <c r="BF27" s="9" t="n"/>
       <c r="BG27" s="9" t="n"/>
       <c r="BH27" s="9" t="n"/>
-      <c r="BI27" s="9" t="n"/>
+      <c r="BI27" s="12" t="n"/>
       <c r="BJ27" s="9" t="n"/>
       <c r="BK27" s="9" t="n"/>
       <c r="BL27" s="9" t="n"/>
       <c r="BM27" s="9" t="n"/>
-      <c r="BN27" s="25" t="inlineStr">
+      <c r="BN27" s="19" t="inlineStr">
         <is>
           <t>了日をもとにマクロを使用して表示</t>
         </is>
@@ -3300,13 +3294,13 @@
       <c r="BQ27" s="9" t="n"/>
       <c r="BR27" s="9" t="n"/>
       <c r="BS27" s="9" t="n"/>
-      <c r="BT27" s="9" t="n"/>
+      <c r="BT27" s="12" t="n"/>
       <c r="BU27" s="9" t="n"/>
       <c r="BV27" s="9" t="n"/>
       <c r="BW27" s="9" t="n"/>
       <c r="BX27" s="9" t="n"/>
       <c r="BY27" s="9" t="n"/>
-      <c r="BZ27" s="9" t="n"/>
+      <c r="BZ27" s="12" t="n"/>
       <c r="CA27" s="9" t="n"/>
       <c r="CB27" s="9" t="n"/>
       <c r="CC27" s="9" t="n"/>
@@ -3317,29 +3311,29 @@
       <c r="CH27" s="9" t="n"/>
       <c r="CI27" s="9" t="n"/>
       <c r="CJ27" s="9" t="n"/>
-      <c r="CK27" s="9" t="n"/>
+      <c r="CK27" s="12" t="n"/>
       <c r="CL27" s="9" t="n"/>
       <c r="CM27" s="9" t="n"/>
       <c r="CN27" s="9" t="n"/>
       <c r="CO27" s="9" t="n"/>
       <c r="CP27" s="9" t="n"/>
-      <c r="CQ27" s="9" t="n"/>
+      <c r="CQ27" s="12" t="n"/>
       <c r="CR27" s="9" t="n"/>
       <c r="CS27" s="9" t="n"/>
       <c r="CT27" s="9" t="n"/>
       <c r="CU27" s="9" t="n"/>
-      <c r="CV27" s="9" t="n"/>
+      <c r="CV27" s="12" t="n"/>
       <c r="CW27" s="9" t="n"/>
       <c r="CX27" s="9" t="n"/>
       <c r="CY27" s="9" t="n"/>
       <c r="CZ27" s="9" t="n"/>
       <c r="DA27" s="9" t="n"/>
-      <c r="DB27" s="9" t="n"/>
+      <c r="DB27" s="12" t="n"/>
       <c r="DC27" s="9" t="n"/>
       <c r="DD27" s="9" t="n"/>
       <c r="DE27" s="9" t="n"/>
       <c r="DF27" s="9" t="n"/>
-      <c r="DG27" s="9" t="n"/>
+      <c r="DG27" s="12" t="n"/>
       <c r="DH27" s="9" t="n"/>
       <c r="DI27" s="9" t="n"/>
       <c r="DJ27" s="9" t="n"/>
@@ -3406,35 +3400,35 @@
           <t>33</t>
         </is>
       </c>
-      <c r="AX28" s="18" t="n"/>
+      <c r="AX28" s="14" t="n"/>
       <c r="AY28" s="13" t="n"/>
       <c r="AZ28" s="13" t="n"/>
       <c r="BA28" s="13" t="n"/>
       <c r="BB28" s="13" t="n"/>
-      <c r="BC28" s="13" t="n"/>
+      <c r="BC28" s="14" t="n"/>
       <c r="BD28" s="13" t="n"/>
       <c r="BE28" s="13" t="n"/>
       <c r="BF28" s="13" t="n"/>
       <c r="BG28" s="13" t="n"/>
       <c r="BH28" s="13" t="n"/>
-      <c r="BI28" s="13" t="n"/>
+      <c r="BI28" s="14" t="n"/>
       <c r="BJ28" s="13" t="n"/>
       <c r="BK28" s="13" t="n"/>
       <c r="BL28" s="13" t="n"/>
       <c r="BM28" s="13" t="n"/>
-      <c r="BN28" s="19" t="n"/>
+      <c r="BN28" s="14" t="n"/>
       <c r="BO28" s="13" t="n"/>
       <c r="BP28" s="13" t="n"/>
       <c r="BQ28" s="13" t="n"/>
       <c r="BR28" s="13" t="n"/>
       <c r="BS28" s="13" t="n"/>
-      <c r="BT28" s="13" t="n"/>
+      <c r="BT28" s="14" t="n"/>
       <c r="BU28" s="13" t="n"/>
       <c r="BV28" s="13" t="n"/>
       <c r="BW28" s="13" t="n"/>
       <c r="BX28" s="13" t="n"/>
       <c r="BY28" s="13" t="n"/>
-      <c r="BZ28" s="13" t="n"/>
+      <c r="BZ28" s="14" t="n"/>
       <c r="CA28" s="13" t="n"/>
       <c r="CB28" s="13" t="n"/>
       <c r="CC28" s="13" t="n"/>
@@ -3449,35 +3443,35 @@
       <c r="CH28" s="13" t="n"/>
       <c r="CI28" s="13" t="n"/>
       <c r="CJ28" s="13" t="n"/>
-      <c r="CK28" s="13" t="n"/>
+      <c r="CK28" s="14" t="n"/>
       <c r="CL28" s="13" t="n"/>
       <c r="CM28" s="13" t="n"/>
       <c r="CN28" s="13" t="n"/>
       <c r="CO28" s="13" t="n"/>
       <c r="CP28" s="13" t="n"/>
-      <c r="CQ28" s="13" t="n"/>
+      <c r="CQ28" s="14" t="n"/>
       <c r="CR28" s="13" t="n"/>
       <c r="CS28" s="13" t="n"/>
       <c r="CT28" s="13" t="n"/>
       <c r="CU28" s="13" t="n"/>
-      <c r="CV28" s="13" t="n"/>
+      <c r="CV28" s="14" t="n"/>
       <c r="CW28" s="13" t="n"/>
       <c r="CX28" s="13" t="n"/>
       <c r="CY28" s="13" t="n"/>
       <c r="CZ28" s="13" t="n"/>
       <c r="DA28" s="13" t="n"/>
-      <c r="DB28" s="13" t="n"/>
+      <c r="DB28" s="14" t="n"/>
       <c r="DC28" s="13" t="n"/>
       <c r="DD28" s="13" t="n"/>
       <c r="DE28" s="13" t="n"/>
       <c r="DF28" s="13" t="n"/>
-      <c r="DG28" s="13" t="n"/>
+      <c r="DG28" s="14" t="n"/>
       <c r="DH28" s="13" t="n"/>
       <c r="DI28" s="13" t="n"/>
       <c r="DJ28" s="13" t="n"/>
       <c r="DK28" s="13" t="n"/>
       <c r="DL28" s="13" t="n"/>
-      <c r="DM28" s="18" t="n"/>
+      <c r="DM28" s="17" t="n"/>
     </row>
     <row r="29" ht="11.34" customHeight="1">
       <c r="H29" s="14" t="n"/>
@@ -3538,35 +3532,35 @@
           <t>59</t>
         </is>
       </c>
-      <c r="AX29" s="10" t="n"/>
+      <c r="AX29" s="12" t="n"/>
       <c r="AY29" s="9" t="n"/>
       <c r="AZ29" s="9" t="n"/>
       <c r="BA29" s="9" t="n"/>
       <c r="BB29" s="9" t="n"/>
-      <c r="BC29" s="9" t="n"/>
+      <c r="BC29" s="12" t="n"/>
       <c r="BD29" s="9" t="n"/>
       <c r="BE29" s="9" t="n"/>
       <c r="BF29" s="9" t="n"/>
       <c r="BG29" s="9" t="n"/>
       <c r="BH29" s="9" t="n"/>
-      <c r="BI29" s="9" t="n"/>
+      <c r="BI29" s="12" t="n"/>
       <c r="BJ29" s="9" t="n"/>
       <c r="BK29" s="9" t="n"/>
       <c r="BL29" s="9" t="n"/>
       <c r="BM29" s="9" t="n"/>
-      <c r="BN29" s="17" t="n"/>
+      <c r="BN29" s="12" t="n"/>
       <c r="BO29" s="9" t="n"/>
       <c r="BP29" s="9" t="n"/>
       <c r="BQ29" s="9" t="n"/>
       <c r="BR29" s="9" t="n"/>
       <c r="BS29" s="9" t="n"/>
-      <c r="BT29" s="9" t="n"/>
+      <c r="BT29" s="12" t="n"/>
       <c r="BU29" s="9" t="n"/>
       <c r="BV29" s="9" t="n"/>
       <c r="BW29" s="9" t="n"/>
       <c r="BX29" s="9" t="n"/>
       <c r="BY29" s="9" t="n"/>
-      <c r="BZ29" s="9" t="n"/>
+      <c r="BZ29" s="12" t="n"/>
       <c r="CA29" s="9" t="n"/>
       <c r="CB29" s="9" t="n"/>
       <c r="CC29" s="9" t="n"/>
@@ -3577,29 +3571,29 @@
       <c r="CH29" s="9" t="n"/>
       <c r="CI29" s="9" t="n"/>
       <c r="CJ29" s="9" t="n"/>
-      <c r="CK29" s="9" t="n"/>
+      <c r="CK29" s="12" t="n"/>
       <c r="CL29" s="9" t="n"/>
       <c r="CM29" s="9" t="n"/>
       <c r="CN29" s="9" t="n"/>
       <c r="CO29" s="9" t="n"/>
       <c r="CP29" s="9" t="n"/>
-      <c r="CQ29" s="9" t="n"/>
+      <c r="CQ29" s="12" t="n"/>
       <c r="CR29" s="9" t="n"/>
       <c r="CS29" s="9" t="n"/>
       <c r="CT29" s="9" t="n"/>
       <c r="CU29" s="9" t="n"/>
-      <c r="CV29" s="9" t="n"/>
+      <c r="CV29" s="12" t="n"/>
       <c r="CW29" s="9" t="n"/>
       <c r="CX29" s="9" t="n"/>
       <c r="CY29" s="9" t="n"/>
       <c r="CZ29" s="9" t="n"/>
       <c r="DA29" s="9" t="n"/>
-      <c r="DB29" s="9" t="n"/>
+      <c r="DB29" s="12" t="n"/>
       <c r="DC29" s="9" t="n"/>
       <c r="DD29" s="9" t="n"/>
       <c r="DE29" s="9" t="n"/>
       <c r="DF29" s="9" t="n"/>
-      <c r="DG29" s="9" t="n"/>
+      <c r="DG29" s="12" t="n"/>
       <c r="DH29" s="9" t="n"/>
       <c r="DI29" s="9" t="n"/>
       <c r="DJ29" s="9" t="n"/>
@@ -3674,35 +3668,35 @@
           <t>69</t>
         </is>
       </c>
-      <c r="AX30" s="18" t="n"/>
+      <c r="AX30" s="14" t="n"/>
       <c r="AY30" s="13" t="n"/>
       <c r="AZ30" s="13" t="n"/>
       <c r="BA30" s="13" t="n"/>
       <c r="BB30" s="13" t="n"/>
-      <c r="BC30" s="13" t="n"/>
+      <c r="BC30" s="14" t="n"/>
       <c r="BD30" s="13" t="n"/>
       <c r="BE30" s="9" t="n"/>
       <c r="BF30" s="9" t="n"/>
       <c r="BG30" s="9" t="n"/>
       <c r="BH30" s="9" t="n"/>
-      <c r="BI30" s="9" t="n"/>
+      <c r="BI30" s="12" t="n"/>
       <c r="BJ30" s="9" t="n"/>
       <c r="BK30" s="9" t="n"/>
       <c r="BL30" s="9" t="n"/>
       <c r="BM30" s="9" t="n"/>
-      <c r="BN30" s="17" t="n"/>
+      <c r="BN30" s="12" t="n"/>
       <c r="BO30" s="9" t="n"/>
       <c r="BP30" s="9" t="n"/>
       <c r="BQ30" s="9" t="n"/>
       <c r="BR30" s="9" t="n"/>
       <c r="BS30" s="13" t="n"/>
-      <c r="BT30" s="13" t="n"/>
+      <c r="BT30" s="14" t="n"/>
       <c r="BU30" s="13" t="n"/>
       <c r="BV30" s="13" t="n"/>
       <c r="BW30" s="13" t="n"/>
       <c r="BX30" s="13" t="n"/>
       <c r="BY30" s="13" t="n"/>
-      <c r="BZ30" s="13" t="n"/>
+      <c r="BZ30" s="14" t="n"/>
       <c r="CA30" s="13" t="n"/>
       <c r="CB30" s="13" t="n"/>
       <c r="CC30" s="13" t="n"/>
@@ -3713,35 +3707,35 @@
       <c r="CH30" s="9" t="n"/>
       <c r="CI30" s="9" t="n"/>
       <c r="CJ30" s="9" t="n"/>
-      <c r="CK30" s="9" t="n"/>
+      <c r="CK30" s="12" t="n"/>
       <c r="CL30" s="9" t="n"/>
       <c r="CM30" s="9" t="n"/>
       <c r="CN30" s="9" t="n"/>
       <c r="CO30" s="9" t="n"/>
       <c r="CP30" s="9" t="n"/>
-      <c r="CQ30" s="9" t="n"/>
+      <c r="CQ30" s="12" t="n"/>
       <c r="CR30" s="13" t="n"/>
       <c r="CS30" s="13" t="n"/>
       <c r="CT30" s="13" t="n"/>
       <c r="CU30" s="13" t="n"/>
-      <c r="CV30" s="13" t="n"/>
+      <c r="CV30" s="14" t="n"/>
       <c r="CW30" s="13" t="n"/>
       <c r="CX30" s="13" t="n"/>
       <c r="CY30" s="13" t="n"/>
       <c r="CZ30" s="13" t="n"/>
       <c r="DA30" s="13" t="n"/>
-      <c r="DB30" s="13" t="n"/>
+      <c r="DB30" s="14" t="n"/>
       <c r="DC30" s="13" t="n"/>
       <c r="DD30" s="13" t="n"/>
       <c r="DE30" s="13" t="n"/>
       <c r="DF30" s="13" t="n"/>
-      <c r="DG30" s="13" t="n"/>
+      <c r="DG30" s="14" t="n"/>
       <c r="DH30" s="13" t="n"/>
       <c r="DI30" s="13" t="n"/>
       <c r="DJ30" s="13" t="n"/>
       <c r="DK30" s="13" t="n"/>
       <c r="DL30" s="13" t="n"/>
-      <c r="DM30" s="18" t="n"/>
+      <c r="DM30" s="17" t="n"/>
     </row>
     <row r="31" ht="11.34" customHeight="1">
       <c r="H31" s="12" t="n"/>
@@ -3802,35 +3796,35 @@
           <t>14</t>
         </is>
       </c>
-      <c r="AX31" s="10" t="n"/>
+      <c r="AX31" s="12" t="n"/>
       <c r="AY31" s="9" t="n"/>
       <c r="AZ31" s="9" t="n"/>
       <c r="BA31" s="9" t="n"/>
       <c r="BB31" s="9" t="n"/>
-      <c r="BC31" s="9" t="n"/>
+      <c r="BC31" s="12" t="n"/>
       <c r="BD31" s="9" t="n"/>
       <c r="BE31" s="9" t="n"/>
       <c r="BF31" s="9" t="n"/>
       <c r="BG31" s="9" t="n"/>
       <c r="BH31" s="9" t="n"/>
-      <c r="BI31" s="9" t="n"/>
+      <c r="BI31" s="12" t="n"/>
       <c r="BJ31" s="9" t="n"/>
       <c r="BK31" s="9" t="n"/>
       <c r="BL31" s="9" t="n"/>
       <c r="BM31" s="9" t="n"/>
-      <c r="BN31" s="17" t="n"/>
+      <c r="BN31" s="12" t="n"/>
       <c r="BO31" s="9" t="n"/>
       <c r="BP31" s="9" t="n"/>
       <c r="BQ31" s="10" t="n"/>
       <c r="BR31" s="9" t="n"/>
       <c r="BS31" s="9" t="n"/>
-      <c r="BT31" s="9" t="n"/>
+      <c r="BT31" s="12" t="n"/>
       <c r="BU31" s="9" t="n"/>
       <c r="BV31" s="9" t="n"/>
       <c r="BW31" s="9" t="n"/>
       <c r="BX31" s="9" t="n"/>
       <c r="BY31" s="9" t="n"/>
-      <c r="BZ31" s="9" t="n"/>
+      <c r="BZ31" s="12" t="n"/>
       <c r="CA31" s="9" t="n"/>
       <c r="CB31" s="9" t="n"/>
       <c r="CC31" s="9" t="n"/>
@@ -3841,29 +3835,29 @@
       <c r="CH31" s="9" t="n"/>
       <c r="CI31" s="9" t="n"/>
       <c r="CJ31" s="9" t="n"/>
-      <c r="CK31" s="9" t="n"/>
+      <c r="CK31" s="12" t="n"/>
       <c r="CL31" s="9" t="n"/>
       <c r="CM31" s="9" t="n"/>
       <c r="CN31" s="9" t="n"/>
       <c r="CO31" s="9" t="n"/>
       <c r="CP31" s="9" t="n"/>
-      <c r="CQ31" s="9" t="n"/>
+      <c r="CQ31" s="12" t="n"/>
       <c r="CR31" s="9" t="n"/>
       <c r="CS31" s="9" t="n"/>
       <c r="CT31" s="9" t="n"/>
       <c r="CU31" s="9" t="n"/>
-      <c r="CV31" s="9" t="n"/>
+      <c r="CV31" s="12" t="n"/>
       <c r="CW31" s="9" t="n"/>
       <c r="CX31" s="9" t="n"/>
       <c r="CY31" s="9" t="n"/>
       <c r="CZ31" s="9" t="n"/>
       <c r="DA31" s="9" t="n"/>
-      <c r="DB31" s="9" t="n"/>
+      <c r="DB31" s="12" t="n"/>
       <c r="DC31" s="9" t="n"/>
       <c r="DD31" s="9" t="n"/>
       <c r="DE31" s="9" t="n"/>
       <c r="DF31" s="9" t="n"/>
-      <c r="DG31" s="9" t="n"/>
+      <c r="DG31" s="12" t="n"/>
       <c r="DH31" s="9" t="n"/>
       <c r="DI31" s="9" t="n"/>
       <c r="DJ31" s="9" t="n"/>
@@ -3942,35 +3936,35 @@
           <t>17</t>
         </is>
       </c>
-      <c r="AX32" s="18" t="n"/>
+      <c r="AX32" s="14" t="n"/>
       <c r="AY32" s="13" t="n"/>
       <c r="AZ32" s="13" t="n"/>
       <c r="BA32" s="13" t="n"/>
       <c r="BB32" s="13" t="n"/>
-      <c r="BC32" s="13" t="n"/>
+      <c r="BC32" s="14" t="n"/>
       <c r="BD32" s="13" t="n"/>
       <c r="BE32" s="13" t="n"/>
       <c r="BF32" s="13" t="n"/>
       <c r="BG32" s="13" t="n"/>
       <c r="BH32" s="13" t="n"/>
-      <c r="BI32" s="13" t="n"/>
+      <c r="BI32" s="14" t="n"/>
       <c r="BJ32" s="13" t="n"/>
       <c r="BK32" s="13" t="n"/>
       <c r="BL32" s="13" t="n"/>
       <c r="BM32" s="13" t="n"/>
-      <c r="BN32" s="17" t="n"/>
+      <c r="BN32" s="12" t="n"/>
       <c r="BO32" s="9" t="n"/>
       <c r="BP32" s="9" t="n"/>
       <c r="BQ32" s="10" t="n"/>
       <c r="BR32" s="9" t="n"/>
       <c r="BS32" s="13" t="n"/>
-      <c r="BT32" s="13" t="n"/>
+      <c r="BT32" s="14" t="n"/>
       <c r="BU32" s="13" t="n"/>
       <c r="BV32" s="13" t="n"/>
       <c r="BW32" s="13" t="n"/>
       <c r="BX32" s="13" t="n"/>
       <c r="BY32" s="13" t="n"/>
-      <c r="BZ32" s="13" t="n"/>
+      <c r="BZ32" s="14" t="n"/>
       <c r="CA32" s="13" t="n"/>
       <c r="CB32" s="13" t="n"/>
       <c r="CC32" s="13" t="n"/>
@@ -3981,35 +3975,35 @@
       <c r="CH32" s="13" t="n"/>
       <c r="CI32" s="13" t="n"/>
       <c r="CJ32" s="13" t="n"/>
-      <c r="CK32" s="13" t="n"/>
+      <c r="CK32" s="14" t="n"/>
       <c r="CL32" s="13" t="n"/>
       <c r="CM32" s="13" t="n"/>
       <c r="CN32" s="13" t="n"/>
       <c r="CO32" s="13" t="n"/>
       <c r="CP32" s="13" t="n"/>
-      <c r="CQ32" s="13" t="n"/>
+      <c r="CQ32" s="14" t="n"/>
       <c r="CR32" s="13" t="n"/>
       <c r="CS32" s="13" t="n"/>
       <c r="CT32" s="13" t="n"/>
       <c r="CU32" s="13" t="n"/>
-      <c r="CV32" s="13" t="n"/>
+      <c r="CV32" s="14" t="n"/>
       <c r="CW32" s="13" t="n"/>
       <c r="CX32" s="13" t="n"/>
       <c r="CY32" s="13" t="n"/>
       <c r="CZ32" s="13" t="n"/>
       <c r="DA32" s="13" t="n"/>
-      <c r="DB32" s="13" t="n"/>
+      <c r="DB32" s="14" t="n"/>
       <c r="DC32" s="13" t="n"/>
       <c r="DD32" s="13" t="n"/>
       <c r="DE32" s="13" t="n"/>
       <c r="DF32" s="13" t="n"/>
-      <c r="DG32" s="13" t="n"/>
+      <c r="DG32" s="14" t="n"/>
       <c r="DH32" s="13" t="n"/>
       <c r="DI32" s="13" t="n"/>
       <c r="DJ32" s="13" t="n"/>
       <c r="DK32" s="13" t="n"/>
       <c r="DL32" s="13" t="n"/>
-      <c r="DM32" s="18" t="n"/>
+      <c r="DM32" s="17" t="n"/>
     </row>
     <row r="33" ht="11.34" customHeight="1">
       <c r="H33" s="14" t="n"/>
@@ -4070,35 +4064,35 @@
           <t>117</t>
         </is>
       </c>
-      <c r="AX33" s="10" t="n"/>
+      <c r="AX33" s="12" t="n"/>
       <c r="AY33" s="9" t="n"/>
       <c r="AZ33" s="9" t="n"/>
       <c r="BA33" s="9" t="n"/>
       <c r="BB33" s="9" t="n"/>
-      <c r="BC33" s="9" t="n"/>
+      <c r="BC33" s="12" t="n"/>
       <c r="BD33" s="9" t="n"/>
       <c r="BE33" s="9" t="n"/>
       <c r="BF33" s="9" t="n"/>
       <c r="BG33" s="9" t="n"/>
       <c r="BH33" s="9" t="n"/>
-      <c r="BI33" s="9" t="n"/>
+      <c r="BI33" s="12" t="n"/>
       <c r="BJ33" s="9" t="n"/>
       <c r="BK33" s="9" t="n"/>
       <c r="BL33" s="9" t="n"/>
       <c r="BM33" s="9" t="n"/>
-      <c r="BN33" s="17" t="n"/>
+      <c r="BN33" s="12" t="n"/>
       <c r="BO33" s="9" t="n"/>
       <c r="BP33" s="9" t="n"/>
       <c r="BQ33" s="10" t="n"/>
       <c r="BR33" s="9" t="n"/>
       <c r="BS33" s="9" t="n"/>
-      <c r="BT33" s="9" t="n"/>
+      <c r="BT33" s="12" t="n"/>
       <c r="BU33" s="9" t="n"/>
       <c r="BV33" s="9" t="n"/>
       <c r="BW33" s="9" t="n"/>
       <c r="BX33" s="9" t="n"/>
       <c r="BY33" s="9" t="n"/>
-      <c r="BZ33" s="9" t="n"/>
+      <c r="BZ33" s="12" t="n"/>
       <c r="CA33" s="9" t="n"/>
       <c r="CB33" s="9" t="n"/>
       <c r="CC33" s="9" t="n"/>
@@ -4109,29 +4103,29 @@
       <c r="CH33" s="9" t="n"/>
       <c r="CI33" s="9" t="n"/>
       <c r="CJ33" s="9" t="n"/>
-      <c r="CK33" s="9" t="n"/>
+      <c r="CK33" s="12" t="n"/>
       <c r="CL33" s="9" t="n"/>
       <c r="CM33" s="9" t="n"/>
       <c r="CN33" s="9" t="n"/>
       <c r="CO33" s="9" t="n"/>
       <c r="CP33" s="9" t="n"/>
-      <c r="CQ33" s="9" t="n"/>
+      <c r="CQ33" s="12" t="n"/>
       <c r="CR33" s="9" t="n"/>
       <c r="CS33" s="9" t="n"/>
       <c r="CT33" s="9" t="n"/>
       <c r="CU33" s="9" t="n"/>
-      <c r="CV33" s="9" t="n"/>
+      <c r="CV33" s="12" t="n"/>
       <c r="CW33" s="9" t="n"/>
       <c r="CX33" s="9" t="n"/>
       <c r="CY33" s="9" t="n"/>
       <c r="CZ33" s="9" t="n"/>
       <c r="DA33" s="9" t="n"/>
-      <c r="DB33" s="9" t="n"/>
+      <c r="DB33" s="12" t="n"/>
       <c r="DC33" s="9" t="n"/>
       <c r="DD33" s="9" t="n"/>
       <c r="DE33" s="9" t="n"/>
       <c r="DF33" s="9" t="n"/>
-      <c r="DG33" s="9" t="n"/>
+      <c r="DG33" s="12" t="n"/>
       <c r="DH33" s="9" t="n"/>
       <c r="DI33" s="9" t="n"/>
       <c r="DJ33" s="9" t="n"/>
@@ -4169,7 +4163,7 @@
       <c r="AD34" s="13" t="n"/>
       <c r="AE34" s="13" t="n"/>
       <c r="AF34" s="13" t="n"/>
-      <c r="AG34" s="26" t="inlineStr">
+      <c r="AG34" s="21" t="inlineStr">
         <is>
           <t>実施中</t>
         </is>
@@ -4198,35 +4192,35 @@
       <c r="AU34" s="13" t="n"/>
       <c r="AV34" s="13" t="n"/>
       <c r="AW34" s="13" t="n"/>
-      <c r="AX34" s="18" t="n"/>
+      <c r="AX34" s="14" t="n"/>
       <c r="AY34" s="13" t="n"/>
       <c r="AZ34" s="13" t="n"/>
       <c r="BA34" s="13" t="n"/>
       <c r="BB34" s="13" t="n"/>
-      <c r="BC34" s="13" t="n"/>
+      <c r="BC34" s="14" t="n"/>
       <c r="BD34" s="13" t="n"/>
       <c r="BE34" s="13" t="n"/>
       <c r="BF34" s="13" t="n"/>
       <c r="BG34" s="13" t="n"/>
       <c r="BH34" s="13" t="n"/>
-      <c r="BI34" s="13" t="n"/>
+      <c r="BI34" s="14" t="n"/>
       <c r="BJ34" s="13" t="n"/>
       <c r="BK34" s="13" t="n"/>
       <c r="BL34" s="13" t="n"/>
       <c r="BM34" s="13" t="n"/>
-      <c r="BN34" s="19" t="n"/>
+      <c r="BN34" s="14" t="n"/>
       <c r="BO34" s="13" t="n"/>
       <c r="BP34" s="13" t="n"/>
       <c r="BQ34" s="10" t="n"/>
       <c r="BR34" s="9" t="n"/>
       <c r="BS34" s="9" t="n"/>
-      <c r="BT34" s="9" t="n"/>
+      <c r="BT34" s="12" t="n"/>
       <c r="BU34" s="9" t="n"/>
       <c r="BV34" s="9" t="n"/>
       <c r="BW34" s="9" t="n"/>
       <c r="BX34" s="9" t="n"/>
       <c r="BY34" s="9" t="n"/>
-      <c r="BZ34" s="9" t="n"/>
+      <c r="BZ34" s="12" t="n"/>
       <c r="CA34" s="9" t="n"/>
       <c r="CB34" s="9" t="n"/>
       <c r="CC34" s="9" t="n"/>
@@ -4237,35 +4231,35 @@
       <c r="CH34" s="9" t="n"/>
       <c r="CI34" s="9" t="n"/>
       <c r="CJ34" s="9" t="n"/>
-      <c r="CK34" s="9" t="n"/>
+      <c r="CK34" s="12" t="n"/>
       <c r="CL34" s="9" t="n"/>
       <c r="CM34" s="9" t="n"/>
       <c r="CN34" s="13" t="n"/>
       <c r="CO34" s="13" t="n"/>
       <c r="CP34" s="13" t="n"/>
-      <c r="CQ34" s="13" t="n"/>
+      <c r="CQ34" s="14" t="n"/>
       <c r="CR34" s="13" t="n"/>
       <c r="CS34" s="13" t="n"/>
       <c r="CT34" s="13" t="n"/>
       <c r="CU34" s="13" t="n"/>
-      <c r="CV34" s="13" t="n"/>
+      <c r="CV34" s="14" t="n"/>
       <c r="CW34" s="13" t="n"/>
       <c r="CX34" s="13" t="n"/>
       <c r="CY34" s="13" t="n"/>
       <c r="CZ34" s="13" t="n"/>
       <c r="DA34" s="13" t="n"/>
-      <c r="DB34" s="13" t="n"/>
+      <c r="DB34" s="14" t="n"/>
       <c r="DC34" s="13" t="n"/>
       <c r="DD34" s="13" t="n"/>
       <c r="DE34" s="13" t="n"/>
       <c r="DF34" s="13" t="n"/>
-      <c r="DG34" s="13" t="n"/>
+      <c r="DG34" s="14" t="n"/>
       <c r="DH34" s="13" t="n"/>
       <c r="DI34" s="13" t="n"/>
       <c r="DJ34" s="13" t="n"/>
       <c r="DK34" s="13" t="n"/>
       <c r="DL34" s="13" t="n"/>
-      <c r="DM34" s="18" t="n"/>
+      <c r="DM34" s="17" t="n"/>
     </row>
     <row r="35" ht="11.34" customHeight="1">
       <c r="H35" s="14" t="n"/>
@@ -4326,35 +4320,35 @@
           <t>41</t>
         </is>
       </c>
-      <c r="AX35" s="10" t="n"/>
+      <c r="AX35" s="12" t="n"/>
       <c r="AY35" s="9" t="n"/>
       <c r="AZ35" s="9" t="n"/>
       <c r="BA35" s="9" t="n"/>
       <c r="BB35" s="9" t="n"/>
-      <c r="BC35" s="9" t="n"/>
+      <c r="BC35" s="12" t="n"/>
       <c r="BD35" s="9" t="n"/>
       <c r="BE35" s="9" t="n"/>
       <c r="BF35" s="9" t="n"/>
       <c r="BG35" s="9" t="n"/>
       <c r="BH35" s="9" t="n"/>
-      <c r="BI35" s="9" t="n"/>
+      <c r="BI35" s="12" t="n"/>
       <c r="BJ35" s="9" t="n"/>
       <c r="BK35" s="9" t="n"/>
       <c r="BL35" s="9" t="n"/>
       <c r="BM35" s="9" t="n"/>
-      <c r="BN35" s="17" t="n"/>
+      <c r="BN35" s="12" t="n"/>
       <c r="BO35" s="9" t="n"/>
       <c r="BP35" s="9" t="n"/>
       <c r="BQ35" s="9" t="n"/>
       <c r="BR35" s="9" t="n"/>
       <c r="BS35" s="9" t="n"/>
-      <c r="BT35" s="9" t="n"/>
+      <c r="BT35" s="12" t="n"/>
       <c r="BU35" s="9" t="n"/>
       <c r="BV35" s="9" t="n"/>
       <c r="BW35" s="9" t="n"/>
       <c r="BX35" s="9" t="n"/>
       <c r="BY35" s="9" t="n"/>
-      <c r="BZ35" s="9" t="n"/>
+      <c r="BZ35" s="12" t="n"/>
       <c r="CA35" s="9" t="n"/>
       <c r="CB35" s="9" t="n"/>
       <c r="CC35" s="9" t="n"/>
@@ -4365,29 +4359,29 @@
       <c r="CH35" s="9" t="n"/>
       <c r="CI35" s="9" t="n"/>
       <c r="CJ35" s="9" t="n"/>
-      <c r="CK35" s="9" t="n"/>
+      <c r="CK35" s="12" t="n"/>
       <c r="CL35" s="9" t="n"/>
       <c r="CM35" s="9" t="n"/>
       <c r="CN35" s="9" t="n"/>
       <c r="CO35" s="9" t="n"/>
       <c r="CP35" s="9" t="n"/>
-      <c r="CQ35" s="9" t="n"/>
+      <c r="CQ35" s="12" t="n"/>
       <c r="CR35" s="9" t="n"/>
       <c r="CS35" s="9" t="n"/>
       <c r="CT35" s="9" t="n"/>
       <c r="CU35" s="9" t="n"/>
-      <c r="CV35" s="9" t="n"/>
+      <c r="CV35" s="12" t="n"/>
       <c r="CW35" s="9" t="n"/>
       <c r="CX35" s="9" t="n"/>
       <c r="CY35" s="9" t="n"/>
       <c r="CZ35" s="9" t="n"/>
       <c r="DA35" s="9" t="n"/>
-      <c r="DB35" s="9" t="n"/>
+      <c r="DB35" s="12" t="n"/>
       <c r="DC35" s="9" t="n"/>
       <c r="DD35" s="9" t="n"/>
       <c r="DE35" s="9" t="n"/>
       <c r="DF35" s="9" t="n"/>
-      <c r="DG35" s="9" t="n"/>
+      <c r="DG35" s="12" t="n"/>
       <c r="DH35" s="9" t="n"/>
       <c r="DI35" s="9" t="n"/>
       <c r="DJ35" s="9" t="n"/>
@@ -4425,7 +4419,7 @@
       <c r="AD36" s="13" t="n"/>
       <c r="AE36" s="13" t="n"/>
       <c r="AF36" s="13" t="n"/>
-      <c r="AG36" s="27" t="inlineStr">
+      <c r="AG36" s="22" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4454,35 +4448,35 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AX36" s="18" t="n"/>
+      <c r="AX36" s="14" t="n"/>
       <c r="AY36" s="13" t="n"/>
       <c r="AZ36" s="13" t="n"/>
       <c r="BA36" s="13" t="n"/>
       <c r="BB36" s="13" t="n"/>
-      <c r="BC36" s="13" t="n"/>
+      <c r="BC36" s="14" t="n"/>
       <c r="BD36" s="13" t="n"/>
       <c r="BE36" s="13" t="n"/>
       <c r="BF36" s="13" t="n"/>
       <c r="BG36" s="13" t="n"/>
       <c r="BH36" s="13" t="n"/>
-      <c r="BI36" s="13" t="n"/>
+      <c r="BI36" s="14" t="n"/>
       <c r="BJ36" s="13" t="n"/>
       <c r="BK36" s="13" t="n"/>
       <c r="BL36" s="13" t="n"/>
       <c r="BM36" s="13" t="n"/>
-      <c r="BN36" s="19" t="n"/>
+      <c r="BN36" s="14" t="n"/>
       <c r="BO36" s="13" t="n"/>
       <c r="BP36" s="13" t="n"/>
       <c r="BQ36" s="13" t="n"/>
       <c r="BR36" s="13" t="n"/>
       <c r="BS36" s="13" t="n"/>
-      <c r="BT36" s="13" t="n"/>
+      <c r="BT36" s="14" t="n"/>
       <c r="BU36" s="13" t="n"/>
       <c r="BV36" s="13" t="n"/>
       <c r="BW36" s="13" t="n"/>
       <c r="BX36" s="13" t="n"/>
       <c r="BY36" s="13" t="n"/>
-      <c r="BZ36" s="13" t="n"/>
+      <c r="BZ36" s="14" t="n"/>
       <c r="CA36" s="13" t="n"/>
       <c r="CB36" s="13" t="n"/>
       <c r="CC36" s="13" t="n"/>
@@ -4493,35 +4487,35 @@
       <c r="CH36" s="13" t="n"/>
       <c r="CI36" s="13" t="n"/>
       <c r="CJ36" s="13" t="n"/>
-      <c r="CK36" s="13" t="n"/>
+      <c r="CK36" s="14" t="n"/>
       <c r="CL36" s="13" t="n"/>
       <c r="CM36" s="9" t="n"/>
       <c r="CN36" s="9" t="n"/>
       <c r="CO36" s="9" t="n"/>
       <c r="CP36" s="9" t="n"/>
-      <c r="CQ36" s="9" t="n"/>
+      <c r="CQ36" s="12" t="n"/>
       <c r="CR36" s="9" t="n"/>
       <c r="CS36" s="9" t="n"/>
       <c r="CT36" s="9" t="n"/>
       <c r="CU36" s="13" t="n"/>
-      <c r="CV36" s="13" t="n"/>
+      <c r="CV36" s="14" t="n"/>
       <c r="CW36" s="13" t="n"/>
       <c r="CX36" s="13" t="n"/>
       <c r="CY36" s="13" t="n"/>
       <c r="CZ36" s="13" t="n"/>
       <c r="DA36" s="13" t="n"/>
-      <c r="DB36" s="13" t="n"/>
+      <c r="DB36" s="14" t="n"/>
       <c r="DC36" s="13" t="n"/>
       <c r="DD36" s="13" t="n"/>
       <c r="DE36" s="13" t="n"/>
       <c r="DF36" s="13" t="n"/>
-      <c r="DG36" s="13" t="n"/>
+      <c r="DG36" s="14" t="n"/>
       <c r="DH36" s="13" t="n"/>
       <c r="DI36" s="13" t="n"/>
       <c r="DJ36" s="13" t="n"/>
       <c r="DK36" s="13" t="n"/>
       <c r="DL36" s="13" t="n"/>
-      <c r="DM36" s="18" t="n"/>
+      <c r="DM36" s="17" t="n"/>
     </row>
     <row r="37" ht="11.34" customHeight="1">
       <c r="H37" s="14" t="n"/>
@@ -4582,35 +4576,35 @@
           <t>41</t>
         </is>
       </c>
-      <c r="AX37" s="10" t="n"/>
+      <c r="AX37" s="12" t="n"/>
       <c r="AY37" s="9" t="n"/>
       <c r="AZ37" s="9" t="n"/>
       <c r="BA37" s="9" t="n"/>
       <c r="BB37" s="9" t="n"/>
-      <c r="BC37" s="9" t="n"/>
+      <c r="BC37" s="12" t="n"/>
       <c r="BD37" s="9" t="n"/>
       <c r="BE37" s="9" t="n"/>
       <c r="BF37" s="9" t="n"/>
       <c r="BG37" s="9" t="n"/>
       <c r="BH37" s="9" t="n"/>
-      <c r="BI37" s="9" t="n"/>
+      <c r="BI37" s="12" t="n"/>
       <c r="BJ37" s="9" t="n"/>
       <c r="BK37" s="9" t="n"/>
       <c r="BL37" s="9" t="n"/>
       <c r="BM37" s="9" t="n"/>
-      <c r="BN37" s="17" t="n"/>
+      <c r="BN37" s="12" t="n"/>
       <c r="BO37" s="9" t="n"/>
       <c r="BP37" s="9" t="n"/>
       <c r="BQ37" s="9" t="n"/>
       <c r="BR37" s="9" t="n"/>
       <c r="BS37" s="9" t="n"/>
-      <c r="BT37" s="9" t="n"/>
+      <c r="BT37" s="12" t="n"/>
       <c r="BU37" s="9" t="n"/>
       <c r="BV37" s="9" t="n"/>
       <c r="BW37" s="9" t="n"/>
       <c r="BX37" s="9" t="n"/>
       <c r="BY37" s="9" t="n"/>
-      <c r="BZ37" s="9" t="n"/>
+      <c r="BZ37" s="12" t="n"/>
       <c r="CA37" s="9" t="n"/>
       <c r="CB37" s="9" t="n"/>
       <c r="CC37" s="9" t="n"/>
@@ -4621,29 +4615,29 @@
       <c r="CH37" s="9" t="n"/>
       <c r="CI37" s="9" t="n"/>
       <c r="CJ37" s="9" t="n"/>
-      <c r="CK37" s="9" t="n"/>
+      <c r="CK37" s="12" t="n"/>
       <c r="CL37" s="9" t="n"/>
       <c r="CM37" s="9" t="n"/>
       <c r="CN37" s="9" t="n"/>
       <c r="CO37" s="9" t="n"/>
       <c r="CP37" s="9" t="n"/>
-      <c r="CQ37" s="9" t="n"/>
+      <c r="CQ37" s="12" t="n"/>
       <c r="CR37" s="9" t="n"/>
       <c r="CS37" s="9" t="n"/>
       <c r="CT37" s="9" t="n"/>
       <c r="CU37" s="9" t="n"/>
-      <c r="CV37" s="9" t="n"/>
+      <c r="CV37" s="12" t="n"/>
       <c r="CW37" s="9" t="n"/>
       <c r="CX37" s="9" t="n"/>
       <c r="CY37" s="9" t="n"/>
       <c r="CZ37" s="9" t="n"/>
       <c r="DA37" s="9" t="n"/>
-      <c r="DB37" s="9" t="n"/>
+      <c r="DB37" s="12" t="n"/>
       <c r="DC37" s="9" t="n"/>
       <c r="DD37" s="9" t="n"/>
       <c r="DE37" s="9" t="n"/>
       <c r="DF37" s="9" t="n"/>
-      <c r="DG37" s="9" t="n"/>
+      <c r="DG37" s="12" t="n"/>
       <c r="DH37" s="9" t="n"/>
       <c r="DI37" s="9" t="n"/>
       <c r="DJ37" s="9" t="n"/>
@@ -4681,7 +4675,7 @@
       <c r="AD38" s="13" t="n"/>
       <c r="AE38" s="13" t="n"/>
       <c r="AF38" s="13" t="n"/>
-      <c r="AG38" s="27" t="inlineStr">
+      <c r="AG38" s="22" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4710,35 +4704,35 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AX38" s="18" t="n"/>
+      <c r="AX38" s="14" t="n"/>
       <c r="AY38" s="13" t="n"/>
       <c r="AZ38" s="13" t="n"/>
       <c r="BA38" s="13" t="n"/>
       <c r="BB38" s="13" t="n"/>
-      <c r="BC38" s="13" t="n"/>
+      <c r="BC38" s="14" t="n"/>
       <c r="BD38" s="13" t="n"/>
       <c r="BE38" s="13" t="n"/>
       <c r="BF38" s="13" t="n"/>
       <c r="BG38" s="13" t="n"/>
       <c r="BH38" s="13" t="n"/>
-      <c r="BI38" s="13" t="n"/>
+      <c r="BI38" s="14" t="n"/>
       <c r="BJ38" s="13" t="n"/>
       <c r="BK38" s="13" t="n"/>
       <c r="BL38" s="13" t="n"/>
       <c r="BM38" s="13" t="n"/>
-      <c r="BN38" s="19" t="n"/>
+      <c r="BN38" s="14" t="n"/>
       <c r="BO38" s="13" t="n"/>
       <c r="BP38" s="13" t="n"/>
       <c r="BQ38" s="13" t="n"/>
       <c r="BR38" s="13" t="n"/>
       <c r="BS38" s="13" t="n"/>
-      <c r="BT38" s="13" t="n"/>
+      <c r="BT38" s="14" t="n"/>
       <c r="BU38" s="13" t="n"/>
       <c r="BV38" s="13" t="n"/>
       <c r="BW38" s="13" t="n"/>
       <c r="BX38" s="13" t="n"/>
       <c r="BY38" s="13" t="n"/>
-      <c r="BZ38" s="13" t="n"/>
+      <c r="BZ38" s="14" t="n"/>
       <c r="CA38" s="13" t="n"/>
       <c r="CB38" s="13" t="n"/>
       <c r="CC38" s="13" t="n"/>
@@ -4749,35 +4743,35 @@
       <c r="CH38" s="13" t="n"/>
       <c r="CI38" s="13" t="n"/>
       <c r="CJ38" s="13" t="n"/>
-      <c r="CK38" s="13" t="n"/>
+      <c r="CK38" s="14" t="n"/>
       <c r="CL38" s="13" t="n"/>
       <c r="CM38" s="9" t="n"/>
       <c r="CN38" s="9" t="n"/>
       <c r="CO38" s="9" t="n"/>
       <c r="CP38" s="9" t="n"/>
-      <c r="CQ38" s="9" t="n"/>
+      <c r="CQ38" s="12" t="n"/>
       <c r="CR38" s="9" t="n"/>
       <c r="CS38" s="9" t="n"/>
       <c r="CT38" s="9" t="n"/>
       <c r="CU38" s="13" t="n"/>
-      <c r="CV38" s="13" t="n"/>
+      <c r="CV38" s="14" t="n"/>
       <c r="CW38" s="13" t="n"/>
       <c r="CX38" s="13" t="n"/>
       <c r="CY38" s="13" t="n"/>
       <c r="CZ38" s="13" t="n"/>
       <c r="DA38" s="13" t="n"/>
-      <c r="DB38" s="13" t="n"/>
+      <c r="DB38" s="14" t="n"/>
       <c r="DC38" s="13" t="n"/>
       <c r="DD38" s="13" t="n"/>
       <c r="DE38" s="13" t="n"/>
       <c r="DF38" s="13" t="n"/>
-      <c r="DG38" s="13" t="n"/>
+      <c r="DG38" s="14" t="n"/>
       <c r="DH38" s="13" t="n"/>
       <c r="DI38" s="13" t="n"/>
       <c r="DJ38" s="13" t="n"/>
       <c r="DK38" s="13" t="n"/>
       <c r="DL38" s="13" t="n"/>
-      <c r="DM38" s="18" t="n"/>
+      <c r="DM38" s="17" t="n"/>
     </row>
     <row r="39" ht="11.34" customHeight="1">
       <c r="H39" s="14" t="n"/>
@@ -4822,35 +4816,35 @@
       <c r="AU39" s="13" t="n"/>
       <c r="AV39" s="13" t="n"/>
       <c r="AW39" s="13" t="n"/>
-      <c r="AX39" s="18" t="n"/>
+      <c r="AX39" s="14" t="n"/>
       <c r="AY39" s="13" t="n"/>
       <c r="AZ39" s="13" t="n"/>
       <c r="BA39" s="13" t="n"/>
       <c r="BB39" s="13" t="n"/>
-      <c r="BC39" s="13" t="n"/>
+      <c r="BC39" s="14" t="n"/>
       <c r="BD39" s="13" t="n"/>
       <c r="BE39" s="13" t="n"/>
       <c r="BF39" s="13" t="n"/>
       <c r="BG39" s="13" t="n"/>
       <c r="BH39" s="13" t="n"/>
-      <c r="BI39" s="13" t="n"/>
+      <c r="BI39" s="14" t="n"/>
       <c r="BJ39" s="13" t="n"/>
       <c r="BK39" s="13" t="n"/>
       <c r="BL39" s="13" t="n"/>
       <c r="BM39" s="13" t="n"/>
-      <c r="BN39" s="19" t="n"/>
+      <c r="BN39" s="14" t="n"/>
       <c r="BO39" s="13" t="n"/>
       <c r="BP39" s="13" t="n"/>
       <c r="BQ39" s="13" t="n"/>
       <c r="BR39" s="13" t="n"/>
       <c r="BS39" s="13" t="n"/>
-      <c r="BT39" s="13" t="n"/>
+      <c r="BT39" s="14" t="n"/>
       <c r="BU39" s="13" t="n"/>
       <c r="BV39" s="13" t="n"/>
       <c r="BW39" s="13" t="n"/>
       <c r="BX39" s="13" t="n"/>
       <c r="BY39" s="13" t="n"/>
-      <c r="BZ39" s="13" t="n"/>
+      <c r="BZ39" s="14" t="n"/>
       <c r="CA39" s="13" t="n"/>
       <c r="CB39" s="13" t="n"/>
       <c r="CC39" s="13" t="n"/>
@@ -4861,35 +4855,35 @@
       <c r="CH39" s="13" t="n"/>
       <c r="CI39" s="13" t="n"/>
       <c r="CJ39" s="13" t="n"/>
-      <c r="CK39" s="13" t="n"/>
+      <c r="CK39" s="14" t="n"/>
       <c r="CL39" s="13" t="n"/>
       <c r="CM39" s="13" t="n"/>
       <c r="CN39" s="13" t="n"/>
       <c r="CO39" s="13" t="n"/>
       <c r="CP39" s="13" t="n"/>
-      <c r="CQ39" s="13" t="n"/>
+      <c r="CQ39" s="14" t="n"/>
       <c r="CR39" s="13" t="n"/>
       <c r="CS39" s="13" t="n"/>
       <c r="CT39" s="13" t="n"/>
       <c r="CU39" s="13" t="n"/>
-      <c r="CV39" s="13" t="n"/>
+      <c r="CV39" s="14" t="n"/>
       <c r="CW39" s="13" t="n"/>
       <c r="CX39" s="13" t="n"/>
       <c r="CY39" s="13" t="n"/>
       <c r="CZ39" s="13" t="n"/>
       <c r="DA39" s="13" t="n"/>
-      <c r="DB39" s="13" t="n"/>
+      <c r="DB39" s="14" t="n"/>
       <c r="DC39" s="13" t="n"/>
       <c r="DD39" s="13" t="n"/>
       <c r="DE39" s="13" t="n"/>
       <c r="DF39" s="13" t="n"/>
-      <c r="DG39" s="13" t="n"/>
+      <c r="DG39" s="14" t="n"/>
       <c r="DH39" s="13" t="n"/>
       <c r="DI39" s="13" t="n"/>
       <c r="DJ39" s="13" t="n"/>
       <c r="DK39" s="13" t="n"/>
       <c r="DL39" s="13" t="n"/>
-      <c r="DM39" s="18" t="n"/>
+      <c r="DM39" s="17" t="n"/>
     </row>
     <row r="40" ht="11.34" customHeight="1">
       <c r="H40" s="16" t="inlineStr">
@@ -4921,7 +4915,7 @@
       <c r="AD40" s="13" t="n"/>
       <c r="AE40" s="13" t="n"/>
       <c r="AF40" s="13" t="n"/>
-      <c r="AG40" s="27" t="inlineStr">
+      <c r="AG40" s="22" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
@@ -4958,35 +4952,35 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AX40" s="18" t="n"/>
+      <c r="AX40" s="14" t="n"/>
       <c r="AY40" s="13" t="n"/>
       <c r="AZ40" s="13" t="n"/>
       <c r="BA40" s="13" t="n"/>
       <c r="BB40" s="13" t="n"/>
-      <c r="BC40" s="13" t="n"/>
+      <c r="BC40" s="14" t="n"/>
       <c r="BD40" s="13" t="n"/>
       <c r="BE40" s="13" t="n"/>
       <c r="BF40" s="13" t="n"/>
       <c r="BG40" s="13" t="n"/>
       <c r="BH40" s="13" t="n"/>
-      <c r="BI40" s="13" t="n"/>
+      <c r="BI40" s="14" t="n"/>
       <c r="BJ40" s="13" t="n"/>
       <c r="BK40" s="13" t="n"/>
       <c r="BL40" s="13" t="n"/>
       <c r="BM40" s="13" t="n"/>
-      <c r="BN40" s="19" t="n"/>
+      <c r="BN40" s="14" t="n"/>
       <c r="BO40" s="13" t="n"/>
       <c r="BP40" s="13" t="n"/>
       <c r="BQ40" s="13" t="n"/>
       <c r="BR40" s="13" t="n"/>
       <c r="BS40" s="13" t="n"/>
-      <c r="BT40" s="13" t="n"/>
+      <c r="BT40" s="14" t="n"/>
       <c r="BU40" s="13" t="n"/>
       <c r="BV40" s="13" t="n"/>
       <c r="BW40" s="13" t="n"/>
       <c r="BX40" s="13" t="n"/>
       <c r="BY40" s="13" t="n"/>
-      <c r="BZ40" s="13" t="n"/>
+      <c r="BZ40" s="14" t="n"/>
       <c r="CA40" s="13" t="n"/>
       <c r="CB40" s="13" t="n"/>
       <c r="CC40" s="13" t="n"/>
@@ -4997,35 +4991,35 @@
       <c r="CH40" s="13" t="n"/>
       <c r="CI40" s="13" t="n"/>
       <c r="CJ40" s="13" t="n"/>
-      <c r="CK40" s="13" t="n"/>
+      <c r="CK40" s="14" t="n"/>
       <c r="CL40" s="13" t="n"/>
       <c r="CM40" s="13" t="n"/>
       <c r="CN40" s="13" t="n"/>
       <c r="CO40" s="13" t="n"/>
       <c r="CP40" s="13" t="n"/>
-      <c r="CQ40" s="13" t="n"/>
+      <c r="CQ40" s="14" t="n"/>
       <c r="CR40" s="13" t="n"/>
       <c r="CS40" s="13" t="n"/>
       <c r="CT40" s="13" t="n"/>
       <c r="CU40" s="13" t="n"/>
-      <c r="CV40" s="9" t="n"/>
+      <c r="CV40" s="12" t="n"/>
       <c r="CW40" s="9" t="n"/>
       <c r="CX40" s="9" t="n"/>
       <c r="CY40" s="9" t="n"/>
       <c r="CZ40" s="9" t="n"/>
       <c r="DA40" s="9" t="n"/>
-      <c r="DB40" s="9" t="n"/>
+      <c r="DB40" s="12" t="n"/>
       <c r="DC40" s="13" t="n"/>
       <c r="DD40" s="13" t="n"/>
       <c r="DE40" s="13" t="n"/>
       <c r="DF40" s="13" t="n"/>
-      <c r="DG40" s="13" t="n"/>
+      <c r="DG40" s="14" t="n"/>
       <c r="DH40" s="13" t="n"/>
       <c r="DI40" s="13" t="n"/>
       <c r="DJ40" s="13" t="n"/>
       <c r="DK40" s="13" t="n"/>
       <c r="DL40" s="13" t="n"/>
-      <c r="DM40" s="18" t="n"/>
+      <c r="DM40" s="17" t="n"/>
     </row>
     <row r="41" ht="11.34" customHeight="1">
       <c r="H41" s="14" t="n"/>
@@ -5070,35 +5064,35 @@
       <c r="AU41" s="13" t="n"/>
       <c r="AV41" s="13" t="n"/>
       <c r="AW41" s="13" t="n"/>
-      <c r="AX41" s="18" t="n"/>
+      <c r="AX41" s="14" t="n"/>
       <c r="AY41" s="13" t="n"/>
       <c r="AZ41" s="13" t="n"/>
       <c r="BA41" s="13" t="n"/>
       <c r="BB41" s="13" t="n"/>
-      <c r="BC41" s="13" t="n"/>
+      <c r="BC41" s="14" t="n"/>
       <c r="BD41" s="13" t="n"/>
       <c r="BE41" s="13" t="n"/>
       <c r="BF41" s="13" t="n"/>
       <c r="BG41" s="13" t="n"/>
       <c r="BH41" s="13" t="n"/>
-      <c r="BI41" s="13" t="n"/>
+      <c r="BI41" s="14" t="n"/>
       <c r="BJ41" s="13" t="n"/>
       <c r="BK41" s="13" t="n"/>
       <c r="BL41" s="13" t="n"/>
       <c r="BM41" s="13" t="n"/>
-      <c r="BN41" s="19" t="n"/>
+      <c r="BN41" s="14" t="n"/>
       <c r="BO41" s="13" t="n"/>
       <c r="BP41" s="13" t="n"/>
       <c r="BQ41" s="13" t="n"/>
       <c r="BR41" s="13" t="n"/>
       <c r="BS41" s="13" t="n"/>
-      <c r="BT41" s="13" t="n"/>
+      <c r="BT41" s="14" t="n"/>
       <c r="BU41" s="13" t="n"/>
       <c r="BV41" s="13" t="n"/>
       <c r="BW41" s="13" t="n"/>
       <c r="BX41" s="13" t="n"/>
       <c r="BY41" s="13" t="n"/>
-      <c r="BZ41" s="13" t="n"/>
+      <c r="BZ41" s="14" t="n"/>
       <c r="CA41" s="13" t="n"/>
       <c r="CB41" s="13" t="n"/>
       <c r="CC41" s="13" t="n"/>
@@ -5109,35 +5103,35 @@
       <c r="CH41" s="13" t="n"/>
       <c r="CI41" s="13" t="n"/>
       <c r="CJ41" s="13" t="n"/>
-      <c r="CK41" s="13" t="n"/>
+      <c r="CK41" s="14" t="n"/>
       <c r="CL41" s="13" t="n"/>
       <c r="CM41" s="13" t="n"/>
       <c r="CN41" s="13" t="n"/>
       <c r="CO41" s="13" t="n"/>
       <c r="CP41" s="13" t="n"/>
-      <c r="CQ41" s="13" t="n"/>
+      <c r="CQ41" s="14" t="n"/>
       <c r="CR41" s="13" t="n"/>
       <c r="CS41" s="13" t="n"/>
       <c r="CT41" s="13" t="n"/>
       <c r="CU41" s="13" t="n"/>
-      <c r="CV41" s="13" t="n"/>
+      <c r="CV41" s="14" t="n"/>
       <c r="CW41" s="13" t="n"/>
       <c r="CX41" s="13" t="n"/>
       <c r="CY41" s="13" t="n"/>
       <c r="CZ41" s="13" t="n"/>
       <c r="DA41" s="13" t="n"/>
-      <c r="DB41" s="13" t="n"/>
+      <c r="DB41" s="14" t="n"/>
       <c r="DC41" s="13" t="n"/>
       <c r="DD41" s="13" t="n"/>
       <c r="DE41" s="13" t="n"/>
       <c r="DF41" s="13" t="n"/>
-      <c r="DG41" s="13" t="n"/>
+      <c r="DG41" s="14" t="n"/>
       <c r="DH41" s="13" t="n"/>
       <c r="DI41" s="13" t="n"/>
       <c r="DJ41" s="13" t="n"/>
       <c r="DK41" s="13" t="n"/>
       <c r="DL41" s="13" t="n"/>
-      <c r="DM41" s="18" t="n"/>
+      <c r="DM41" s="17" t="n"/>
     </row>
     <row r="42" ht="11.34" customHeight="1">
       <c r="H42" s="8" t="inlineStr">
@@ -5169,7 +5163,7 @@
       <c r="AD42" s="9" t="n"/>
       <c r="AE42" s="9" t="n"/>
       <c r="AF42" s="9" t="n"/>
-      <c r="AG42" s="23" t="inlineStr">
+      <c r="AG42" s="20" t="inlineStr">
         <is>
           <t>実施中</t>
         </is>
@@ -5198,35 +5192,35 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AX42" s="10" t="n"/>
+      <c r="AX42" s="12" t="n"/>
       <c r="AY42" s="9" t="n"/>
       <c r="AZ42" s="9" t="n"/>
       <c r="BA42" s="9" t="n"/>
       <c r="BB42" s="9" t="n"/>
-      <c r="BC42" s="9" t="n"/>
+      <c r="BC42" s="12" t="n"/>
       <c r="BD42" s="9" t="n"/>
       <c r="BE42" s="9" t="n"/>
       <c r="BF42" s="9" t="n"/>
       <c r="BG42" s="9" t="n"/>
       <c r="BH42" s="9" t="n"/>
-      <c r="BI42" s="9" t="n"/>
+      <c r="BI42" s="12" t="n"/>
       <c r="BJ42" s="9" t="n"/>
       <c r="BK42" s="9" t="n"/>
       <c r="BL42" s="9" t="n"/>
       <c r="BM42" s="9" t="n"/>
-      <c r="BN42" s="17" t="n"/>
+      <c r="BN42" s="12" t="n"/>
       <c r="BO42" s="9" t="n"/>
       <c r="BP42" s="9" t="n"/>
       <c r="BQ42" s="9" t="n"/>
       <c r="BR42" s="9" t="n"/>
       <c r="BS42" s="9" t="n"/>
-      <c r="BT42" s="9" t="n"/>
+      <c r="BT42" s="12" t="n"/>
       <c r="BU42" s="9" t="n"/>
       <c r="BV42" s="9" t="n"/>
       <c r="BW42" s="9" t="n"/>
       <c r="BX42" s="9" t="n"/>
       <c r="BY42" s="9" t="n"/>
-      <c r="BZ42" s="9" t="n"/>
+      <c r="BZ42" s="12" t="n"/>
       <c r="CA42" s="9" t="n"/>
       <c r="CB42" s="9" t="n"/>
       <c r="CC42" s="9" t="n"/>
@@ -5237,29 +5231,29 @@
       <c r="CH42" s="9" t="n"/>
       <c r="CI42" s="9" t="n"/>
       <c r="CJ42" s="9" t="n"/>
-      <c r="CK42" s="9" t="n"/>
+      <c r="CK42" s="12" t="n"/>
       <c r="CL42" s="9" t="n"/>
       <c r="CM42" s="9" t="n"/>
       <c r="CN42" s="9" t="n"/>
       <c r="CO42" s="9" t="n"/>
       <c r="CP42" s="9" t="n"/>
-      <c r="CQ42" s="9" t="n"/>
+      <c r="CQ42" s="12" t="n"/>
       <c r="CR42" s="9" t="n"/>
       <c r="CS42" s="9" t="n"/>
       <c r="CT42" s="9" t="n"/>
       <c r="CU42" s="9" t="n"/>
-      <c r="CV42" s="9" t="n"/>
+      <c r="CV42" s="12" t="n"/>
       <c r="CW42" s="9" t="n"/>
       <c r="CX42" s="9" t="n"/>
       <c r="CY42" s="9" t="n"/>
       <c r="CZ42" s="9" t="n"/>
       <c r="DA42" s="9" t="n"/>
-      <c r="DB42" s="9" t="n"/>
+      <c r="DB42" s="12" t="n"/>
       <c r="DC42" s="9" t="n"/>
       <c r="DD42" s="9" t="n"/>
       <c r="DE42" s="9" t="n"/>
       <c r="DF42" s="9" t="n"/>
-      <c r="DG42" s="9" t="n"/>
+      <c r="DG42" s="12" t="n"/>
       <c r="DH42" s="9" t="n"/>
       <c r="DI42" s="9" t="n"/>
       <c r="DJ42" s="9" t="n"/>
@@ -5318,35 +5312,35 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AX43" s="18" t="n"/>
+      <c r="AX43" s="14" t="n"/>
       <c r="AY43" s="13" t="n"/>
       <c r="AZ43" s="13" t="n"/>
       <c r="BA43" s="13" t="n"/>
       <c r="BB43" s="13" t="n"/>
-      <c r="BC43" s="13" t="n"/>
+      <c r="BC43" s="14" t="n"/>
       <c r="BD43" s="13" t="n"/>
       <c r="BE43" s="13" t="n"/>
       <c r="BF43" s="13" t="n"/>
       <c r="BG43" s="13" t="n"/>
       <c r="BH43" s="13" t="n"/>
-      <c r="BI43" s="13" t="n"/>
+      <c r="BI43" s="14" t="n"/>
       <c r="BJ43" s="13" t="n"/>
       <c r="BK43" s="13" t="n"/>
       <c r="BL43" s="13" t="n"/>
       <c r="BM43" s="13" t="n"/>
-      <c r="BN43" s="19" t="n"/>
+      <c r="BN43" s="14" t="n"/>
       <c r="BO43" s="13" t="n"/>
       <c r="BP43" s="13" t="n"/>
       <c r="BQ43" s="13" t="n"/>
       <c r="BR43" s="9" t="n"/>
       <c r="BS43" s="9" t="n"/>
-      <c r="BT43" s="9" t="n"/>
+      <c r="BT43" s="12" t="n"/>
       <c r="BU43" s="13" t="n"/>
       <c r="BV43" s="13" t="n"/>
       <c r="BW43" s="13" t="n"/>
       <c r="BX43" s="13" t="n"/>
       <c r="BY43" s="13" t="n"/>
-      <c r="BZ43" s="13" t="n"/>
+      <c r="BZ43" s="14" t="n"/>
       <c r="CA43" s="13" t="n"/>
       <c r="CB43" s="13" t="n"/>
       <c r="CC43" s="13" t="n"/>
@@ -5357,35 +5351,35 @@
       <c r="CH43" s="13" t="n"/>
       <c r="CI43" s="13" t="n"/>
       <c r="CJ43" s="13" t="n"/>
-      <c r="CK43" s="13" t="n"/>
+      <c r="CK43" s="14" t="n"/>
       <c r="CL43" s="13" t="n"/>
       <c r="CM43" s="13" t="n"/>
       <c r="CN43" s="13" t="n"/>
       <c r="CO43" s="13" t="n"/>
       <c r="CP43" s="13" t="n"/>
-      <c r="CQ43" s="13" t="n"/>
+      <c r="CQ43" s="14" t="n"/>
       <c r="CR43" s="13" t="n"/>
       <c r="CS43" s="13" t="n"/>
       <c r="CT43" s="13" t="n"/>
       <c r="CU43" s="13" t="n"/>
-      <c r="CV43" s="13" t="n"/>
+      <c r="CV43" s="14" t="n"/>
       <c r="CW43" s="13" t="n"/>
       <c r="CX43" s="13" t="n"/>
       <c r="CY43" s="13" t="n"/>
       <c r="CZ43" s="13" t="n"/>
       <c r="DA43" s="13" t="n"/>
-      <c r="DB43" s="13" t="n"/>
+      <c r="DB43" s="14" t="n"/>
       <c r="DC43" s="13" t="n"/>
       <c r="DD43" s="13" t="n"/>
       <c r="DE43" s="13" t="n"/>
       <c r="DF43" s="13" t="n"/>
-      <c r="DG43" s="13" t="n"/>
+      <c r="DG43" s="14" t="n"/>
       <c r="DH43" s="13" t="n"/>
       <c r="DI43" s="13" t="n"/>
       <c r="DJ43" s="13" t="n"/>
       <c r="DK43" s="13" t="n"/>
       <c r="DL43" s="13" t="n"/>
-      <c r="DM43" s="18" t="n"/>
+      <c r="DM43" s="17" t="n"/>
     </row>
     <row r="44" ht="11.34" customHeight="1">
       <c r="H44" s="14" t="n"/>
@@ -5430,35 +5424,35 @@
       <c r="AU44" s="13" t="n"/>
       <c r="AV44" s="13" t="n"/>
       <c r="AW44" s="13" t="n"/>
-      <c r="AX44" s="18" t="n"/>
+      <c r="AX44" s="14" t="n"/>
       <c r="AY44" s="13" t="n"/>
       <c r="AZ44" s="13" t="n"/>
       <c r="BA44" s="13" t="n"/>
       <c r="BB44" s="13" t="n"/>
-      <c r="BC44" s="13" t="n"/>
+      <c r="BC44" s="14" t="n"/>
       <c r="BD44" s="13" t="n"/>
       <c r="BE44" s="13" t="n"/>
       <c r="BF44" s="13" t="n"/>
       <c r="BG44" s="13" t="n"/>
       <c r="BH44" s="13" t="n"/>
-      <c r="BI44" s="13" t="n"/>
+      <c r="BI44" s="14" t="n"/>
       <c r="BJ44" s="13" t="n"/>
       <c r="BK44" s="13" t="n"/>
       <c r="BL44" s="13" t="n"/>
       <c r="BM44" s="13" t="n"/>
-      <c r="BN44" s="19" t="n"/>
+      <c r="BN44" s="14" t="n"/>
       <c r="BO44" s="13" t="n"/>
       <c r="BP44" s="13" t="n"/>
       <c r="BQ44" s="13" t="n"/>
       <c r="BR44" s="13" t="n"/>
       <c r="BS44" s="13" t="n"/>
-      <c r="BT44" s="13" t="n"/>
+      <c r="BT44" s="14" t="n"/>
       <c r="BU44" s="13" t="n"/>
       <c r="BV44" s="13" t="n"/>
       <c r="BW44" s="13" t="n"/>
       <c r="BX44" s="13" t="n"/>
       <c r="BY44" s="13" t="n"/>
-      <c r="BZ44" s="13" t="n"/>
+      <c r="BZ44" s="14" t="n"/>
       <c r="CA44" s="13" t="n"/>
       <c r="CB44" s="13" t="n"/>
       <c r="CC44" s="13" t="n"/>
@@ -5469,35 +5463,35 @@
       <c r="CH44" s="13" t="n"/>
       <c r="CI44" s="13" t="n"/>
       <c r="CJ44" s="13" t="n"/>
-      <c r="CK44" s="13" t="n"/>
+      <c r="CK44" s="14" t="n"/>
       <c r="CL44" s="13" t="n"/>
       <c r="CM44" s="13" t="n"/>
       <c r="CN44" s="13" t="n"/>
       <c r="CO44" s="13" t="n"/>
       <c r="CP44" s="13" t="n"/>
-      <c r="CQ44" s="13" t="n"/>
+      <c r="CQ44" s="14" t="n"/>
       <c r="CR44" s="13" t="n"/>
       <c r="CS44" s="13" t="n"/>
       <c r="CT44" s="13" t="n"/>
       <c r="CU44" s="13" t="n"/>
-      <c r="CV44" s="13" t="n"/>
+      <c r="CV44" s="14" t="n"/>
       <c r="CW44" s="13" t="n"/>
       <c r="CX44" s="13" t="n"/>
       <c r="CY44" s="13" t="n"/>
       <c r="CZ44" s="13" t="n"/>
       <c r="DA44" s="13" t="n"/>
-      <c r="DB44" s="13" t="n"/>
+      <c r="DB44" s="14" t="n"/>
       <c r="DC44" s="13" t="n"/>
       <c r="DD44" s="13" t="n"/>
       <c r="DE44" s="13" t="n"/>
       <c r="DF44" s="13" t="n"/>
-      <c r="DG44" s="13" t="n"/>
+      <c r="DG44" s="14" t="n"/>
       <c r="DH44" s="13" t="n"/>
       <c r="DI44" s="13" t="n"/>
       <c r="DJ44" s="13" t="n"/>
       <c r="DK44" s="13" t="n"/>
       <c r="DL44" s="13" t="n"/>
-      <c r="DM44" s="18" t="n"/>
+      <c r="DM44" s="17" t="n"/>
     </row>
     <row r="45" ht="11.34" customHeight="1">
       <c r="H45" s="12" t="n"/>
@@ -5512,8 +5506,8 @@
       <c r="M45" s="9" t="n"/>
       <c r="N45" s="9" t="n"/>
       <c r="O45" s="12" t="n"/>
-      <c r="T45" s="28" t="n"/>
-      <c r="U45" s="29" t="inlineStr">
+      <c r="T45" s="23" t="n"/>
+      <c r="U45" s="24" t="inlineStr">
         <is>
           <t>必要に応じて行を追加</t>
         </is>
@@ -5529,10 +5523,10 @@
       <c r="AD45" s="6" t="n"/>
       <c r="AE45" s="6" t="n"/>
       <c r="AF45" s="7" t="n"/>
-      <c r="AX45" s="28" t="n"/>
+      <c r="AX45" s="23" t="n"/>
       <c r="AY45" s="6" t="n"/>
       <c r="AZ45" s="6" t="n"/>
-      <c r="BA45" s="30" t="inlineStr">
+      <c r="BA45" s="25" t="inlineStr">
         <is>
           <t>計画</t>
         </is>
@@ -5547,7 +5541,7 @@
       <c r="M46" s="9" t="n"/>
       <c r="N46" s="9" t="n"/>
       <c r="O46" s="12" t="n"/>
-      <c r="T46" s="19" t="n"/>
+      <c r="T46" s="26" t="n"/>
       <c r="U46" s="13" t="n"/>
       <c r="V46" s="13" t="n"/>
       <c r="W46" s="13" t="n"/>
@@ -5559,37 +5553,37 @@
       <c r="AC46" s="13" t="n"/>
       <c r="AD46" s="13" t="n"/>
       <c r="AE46" s="13" t="n"/>
-      <c r="AF46" s="18" t="n"/>
-      <c r="AX46" s="17" t="n"/>
+      <c r="AF46" s="17" t="n"/>
+      <c r="AX46" s="27" t="n"/>
       <c r="AY46" s="9" t="n"/>
       <c r="AZ46" s="9" t="n"/>
-      <c r="BA46" s="31" t="inlineStr">
+      <c r="BA46" s="28" t="inlineStr">
         <is>
           <t>実績</t>
         </is>
       </c>
     </row>
     <row r="47" ht="11.34" customHeight="1">
-      <c r="T47" s="32" t="n"/>
-      <c r="U47" s="33" t="n"/>
-      <c r="V47" s="33" t="n"/>
-      <c r="W47" s="33" t="n"/>
-      <c r="X47" s="33" t="n"/>
-      <c r="Y47" s="33" t="n"/>
-      <c r="Z47" s="33" t="n"/>
-      <c r="AA47" s="33" t="n"/>
-      <c r="AB47" s="33" t="n"/>
-      <c r="AC47" s="33" t="n"/>
-      <c r="AD47" s="33" t="n"/>
-      <c r="AE47" s="33" t="n"/>
-      <c r="AF47" s="34" t="n"/>
-      <c r="AX47" s="32" t="n"/>
-      <c r="AY47" s="33" t="n"/>
-      <c r="AZ47" s="33" t="n"/>
-      <c r="BA47" s="34" t="n"/>
+      <c r="T47" s="29" t="n"/>
+      <c r="U47" s="30" t="n"/>
+      <c r="V47" s="30" t="n"/>
+      <c r="W47" s="30" t="n"/>
+      <c r="X47" s="30" t="n"/>
+      <c r="Y47" s="30" t="n"/>
+      <c r="Z47" s="30" t="n"/>
+      <c r="AA47" s="30" t="n"/>
+      <c r="AB47" s="30" t="n"/>
+      <c r="AC47" s="30" t="n"/>
+      <c r="AD47" s="30" t="n"/>
+      <c r="AE47" s="30" t="n"/>
+      <c r="AF47" s="31" t="n"/>
+      <c r="AX47" s="29" t="n"/>
+      <c r="AY47" s="30" t="n"/>
+      <c r="AZ47" s="30" t="n"/>
+      <c r="BA47" s="31" t="n"/>
     </row>
     <row r="48" ht="11.34" customHeight="1">
-      <c r="H48" s="35" t="inlineStr">
+      <c r="H48" s="32" t="inlineStr">
         <is>
           <t>【3.作業事項及び対応状況等】</t>
         </is>
@@ -5638,7 +5632,7 @@
       <c r="AX48" s="6" t="n"/>
       <c r="AY48" s="6" t="n"/>
       <c r="AZ48" s="6" t="n"/>
-      <c r="BA48" s="36" t="n"/>
+      <c r="BA48" s="33" t="n"/>
       <c r="BB48" s="6" t="n"/>
       <c r="BC48" s="6" t="n"/>
       <c r="BD48" s="6" t="n"/>
@@ -5664,7 +5658,7 @@
         </is>
       </c>
       <c r="I49" s="9" t="n"/>
-      <c r="J49" s="17" t="n"/>
+      <c r="J49" s="27" t="n"/>
       <c r="K49" s="9" t="n"/>
       <c r="L49" s="9" t="n"/>
       <c r="M49" s="9" t="n"/>
@@ -5769,7 +5763,7 @@
         </is>
       </c>
       <c r="I50" s="9" t="n"/>
-      <c r="J50" s="24" t="inlineStr">
+      <c r="J50" s="34" t="inlineStr">
         <is>
           <t>着手時、経歴書、技術者届等</t>
         </is>
@@ -5862,7 +5856,7 @@
         </is>
       </c>
       <c r="I51" s="9" t="n"/>
-      <c r="J51" s="24" t="inlineStr">
+      <c r="J51" s="34" t="inlineStr">
         <is>
           <t>業務計画書作成</t>
         </is>
@@ -5951,7 +5945,7 @@
     <row r="52" ht="11.34" customHeight="1">
       <c r="H52" s="12" t="n"/>
       <c r="I52" s="9" t="n"/>
-      <c r="J52" s="17" t="n"/>
+      <c r="J52" s="27" t="n"/>
       <c r="K52" s="9" t="n"/>
       <c r="L52" s="9" t="n"/>
       <c r="M52" s="9" t="n"/>
@@ -6020,7 +6014,7 @@
         </is>
       </c>
       <c r="I53" s="9" t="n"/>
-      <c r="J53" s="24" t="inlineStr">
+      <c r="J53" s="34" t="inlineStr">
         <is>
           <t>交通量配分用データの作成</t>
         </is>
@@ -6109,7 +6103,7 @@
     <row r="54" ht="11.34" customHeight="1">
       <c r="H54" s="12" t="n"/>
       <c r="I54" s="9" t="n"/>
-      <c r="J54" s="17" t="n"/>
+      <c r="J54" s="27" t="n"/>
       <c r="K54" s="9" t="n"/>
       <c r="L54" s="9" t="n"/>
       <c r="M54" s="9" t="n"/>
@@ -6174,7 +6168,7 @@
     <row r="55" ht="11.34" customHeight="1">
       <c r="H55" s="12" t="n"/>
       <c r="I55" s="9" t="n"/>
-      <c r="J55" s="17" t="n"/>
+      <c r="J55" s="27" t="n"/>
       <c r="K55" s="9" t="n"/>
       <c r="L55" s="9" t="n"/>
       <c r="M55" s="9" t="n"/>
@@ -6239,7 +6233,7 @@
     <row r="56" ht="11.34" customHeight="1">
       <c r="H56" s="12" t="n"/>
       <c r="I56" s="9" t="n"/>
-      <c r="J56" s="17" t="n"/>
+      <c r="J56" s="27" t="n"/>
       <c r="K56" s="9" t="n"/>
       <c r="L56" s="9" t="n"/>
       <c r="M56" s="9" t="n"/>
@@ -6304,7 +6298,7 @@
     <row r="57" ht="11.34" customHeight="1">
       <c r="H57" s="12" t="n"/>
       <c r="I57" s="9" t="n"/>
-      <c r="J57" s="17" t="n"/>
+      <c r="J57" s="27" t="n"/>
       <c r="K57" s="9" t="n"/>
       <c r="L57" s="9" t="n"/>
       <c r="M57" s="9" t="n"/>
@@ -6367,72 +6361,72 @@
       <c r="BR57" s="10" t="n"/>
     </row>
     <row r="58" ht="11.34" customHeight="1">
-      <c r="H58" s="37" t="n"/>
-      <c r="I58" s="33" t="n"/>
-      <c r="J58" s="32" t="n"/>
-      <c r="K58" s="33" t="n"/>
-      <c r="L58" s="33" t="n"/>
-      <c r="M58" s="33" t="n"/>
-      <c r="N58" s="33" t="n"/>
-      <c r="O58" s="33" t="n"/>
-      <c r="P58" s="33" t="n"/>
-      <c r="Q58" s="33" t="n"/>
-      <c r="R58" s="33" t="n"/>
-      <c r="S58" s="33" t="n"/>
-      <c r="T58" s="33" t="n"/>
-      <c r="U58" s="33" t="n"/>
-      <c r="V58" s="33" t="n"/>
-      <c r="W58" s="33" t="n"/>
-      <c r="X58" s="33" t="n"/>
-      <c r="Y58" s="33" t="n"/>
-      <c r="Z58" s="33" t="n"/>
-      <c r="AA58" s="33" t="n"/>
-      <c r="AB58" s="33" t="n"/>
-      <c r="AC58" s="33" t="n"/>
-      <c r="AD58" s="33" t="n"/>
-      <c r="AE58" s="33" t="n"/>
-      <c r="AF58" s="33" t="n"/>
-      <c r="AG58" s="37" t="n"/>
-      <c r="AH58" s="33" t="n"/>
-      <c r="AI58" s="33" t="n"/>
-      <c r="AJ58" s="37" t="n"/>
-      <c r="AK58" s="33" t="n"/>
-      <c r="AL58" s="33" t="n"/>
-      <c r="AM58" s="37" t="n"/>
-      <c r="AN58" s="33" t="n"/>
-      <c r="AO58" s="33" t="n"/>
-      <c r="AP58" s="33" t="n"/>
-      <c r="AQ58" s="37" t="n"/>
-      <c r="AR58" s="33" t="n"/>
-      <c r="AS58" s="33" t="n"/>
-      <c r="AT58" s="37" t="n"/>
-      <c r="AU58" s="33" t="n"/>
-      <c r="AV58" s="33" t="n"/>
-      <c r="AW58" s="33" t="n"/>
-      <c r="AX58" s="37" t="n"/>
-      <c r="AY58" s="33" t="n"/>
-      <c r="AZ58" s="33" t="n"/>
-      <c r="BA58" s="37" t="n"/>
-      <c r="BB58" s="33" t="n"/>
-      <c r="BC58" s="33" t="n"/>
-      <c r="BD58" s="33" t="n"/>
-      <c r="BE58" s="33" t="n"/>
-      <c r="BF58" s="33" t="n"/>
-      <c r="BG58" s="33" t="n"/>
-      <c r="BH58" s="33" t="n"/>
-      <c r="BI58" s="33" t="n"/>
-      <c r="BJ58" s="33" t="n"/>
-      <c r="BK58" s="33" t="n"/>
-      <c r="BL58" s="33" t="n"/>
-      <c r="BM58" s="33" t="n"/>
-      <c r="BN58" s="33" t="n"/>
-      <c r="BO58" s="33" t="n"/>
-      <c r="BP58" s="33" t="n"/>
-      <c r="BQ58" s="33" t="n"/>
-      <c r="BR58" s="34" t="n"/>
+      <c r="H58" s="35" t="n"/>
+      <c r="I58" s="30" t="n"/>
+      <c r="J58" s="29" t="n"/>
+      <c r="K58" s="30" t="n"/>
+      <c r="L58" s="30" t="n"/>
+      <c r="M58" s="30" t="n"/>
+      <c r="N58" s="30" t="n"/>
+      <c r="O58" s="30" t="n"/>
+      <c r="P58" s="30" t="n"/>
+      <c r="Q58" s="30" t="n"/>
+      <c r="R58" s="30" t="n"/>
+      <c r="S58" s="30" t="n"/>
+      <c r="T58" s="30" t="n"/>
+      <c r="U58" s="30" t="n"/>
+      <c r="V58" s="30" t="n"/>
+      <c r="W58" s="30" t="n"/>
+      <c r="X58" s="30" t="n"/>
+      <c r="Y58" s="30" t="n"/>
+      <c r="Z58" s="30" t="n"/>
+      <c r="AA58" s="30" t="n"/>
+      <c r="AB58" s="30" t="n"/>
+      <c r="AC58" s="30" t="n"/>
+      <c r="AD58" s="30" t="n"/>
+      <c r="AE58" s="30" t="n"/>
+      <c r="AF58" s="30" t="n"/>
+      <c r="AG58" s="35" t="n"/>
+      <c r="AH58" s="30" t="n"/>
+      <c r="AI58" s="30" t="n"/>
+      <c r="AJ58" s="35" t="n"/>
+      <c r="AK58" s="30" t="n"/>
+      <c r="AL58" s="30" t="n"/>
+      <c r="AM58" s="35" t="n"/>
+      <c r="AN58" s="30" t="n"/>
+      <c r="AO58" s="30" t="n"/>
+      <c r="AP58" s="30" t="n"/>
+      <c r="AQ58" s="35" t="n"/>
+      <c r="AR58" s="30" t="n"/>
+      <c r="AS58" s="30" t="n"/>
+      <c r="AT58" s="35" t="n"/>
+      <c r="AU58" s="30" t="n"/>
+      <c r="AV58" s="30" t="n"/>
+      <c r="AW58" s="30" t="n"/>
+      <c r="AX58" s="35" t="n"/>
+      <c r="AY58" s="30" t="n"/>
+      <c r="AZ58" s="30" t="n"/>
+      <c r="BA58" s="35" t="n"/>
+      <c r="BB58" s="30" t="n"/>
+      <c r="BC58" s="30" t="n"/>
+      <c r="BD58" s="30" t="n"/>
+      <c r="BE58" s="30" t="n"/>
+      <c r="BF58" s="30" t="n"/>
+      <c r="BG58" s="30" t="n"/>
+      <c r="BH58" s="30" t="n"/>
+      <c r="BI58" s="30" t="n"/>
+      <c r="BJ58" s="30" t="n"/>
+      <c r="BK58" s="30" t="n"/>
+      <c r="BL58" s="30" t="n"/>
+      <c r="BM58" s="30" t="n"/>
+      <c r="BN58" s="30" t="n"/>
+      <c r="BO58" s="30" t="n"/>
+      <c r="BP58" s="30" t="n"/>
+      <c r="BQ58" s="30" t="n"/>
+      <c r="BR58" s="31" t="n"/>
     </row>
     <row r="59" ht="11.34" customHeight="1">
-      <c r="H59" s="37" t="n"/>
+      <c r="H59" s="35" t="n"/>
     </row>
     <row r="60" ht="11.34" customHeight="1"/>
     <row r="61" ht="11.34" customHeight="1"/>

</xml_diff>